<commit_message>
Add Music sheet to the Memory Lane reel workbook
Adds a fifth sheet with audio-picker search terms, calm/nostalgic track
picks, the native-audio posting rules, and a sync note tying the track's
swell to the orb-fill shot.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JLTsBRbD5LTCiR7DCK43kP
</commit_message>
<xml_diff>
--- a/memory-lane-reel.xlsx
+++ b/memory-lane-reel.xlsx
@@ -11,6 +11,7 @@
     <sheet name="How to Record" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Edit Steps" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Post" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Music" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1420,4 +1421,226 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Music</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Calm, warm, slightly nostalgic, building gently. Softer than a launch hype edit. Add it INSIDE Instagram, mute your export.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="24" t="inlineStr">
+        <is>
+          <t>Search these in the Reels audio picker</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Search term</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>What it pulls</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="23" t="inlineStr">
+        <is>
+          <t>aesthetic / calm aesthetic</t>
+        </is>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>the soft instrumental lane</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="23" t="inlineStr">
+        <is>
+          <t>nostalgic</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>wistful, looking-back tracks</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>slowed + reverb</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>slowed edits of a song you like — big for this mood</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="24" t="inlineStr">
+        <is>
+          <t>Tracks usually available in this space</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Track</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Feel</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="23" t="inlineStr">
+        <is>
+          <t>Snowfall — Oneheart &amp; reidenshi</t>
+        </is>
+      </c>
+      <c r="B11" s="22" t="inlineStr">
+        <is>
+          <t>soft, spacious, the default calm-reel sound</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="23" t="inlineStr">
+        <is>
+          <t>Until I Found You (piano / slowed)</t>
+        </is>
+      </c>
+      <c r="B12" s="22" t="inlineStr">
+        <is>
+          <t>warm, emotional, builds gently</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="23" t="inlineStr">
+        <is>
+          <t>Glimpse of Us — Joji (instrumental)</t>
+        </is>
+      </c>
+      <c r="B13" s="22" t="inlineStr">
+        <is>
+          <t>nostalgic, piano-led</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1">
+      <c r="A14" s="23" t="inlineStr">
+        <is>
+          <t>Ludovico Einaudi — Nuvole Bianche</t>
+        </is>
+      </c>
+      <c r="B14" s="22" t="inlineStr">
+        <is>
+          <t>pure emotion, no lyrics to fight your text</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="23" t="inlineStr">
+        <is>
+          <t>lo-fi study / chill loops</t>
+        </is>
+      </c>
+      <c r="B15" s="22" t="inlineStr">
+        <is>
+          <t>safe, calm, endlessly available</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="24" t="inlineStr">
+        <is>
+          <t>The rules that matter more than the exact song</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="25" t="inlineStr">
+        <is>
+          <t>1. Pick a track with a SOFT BEAT, not pure ambient — your cuts need something to land on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="25" t="inlineStr">
+        <is>
+          <t>2. Choose the version with the most reels attached (the number under it). That's the discovery signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="25" t="inlineStr">
+        <is>
+          <t>3. Instrumental / no lyrics, so the music never competes with your on-screen text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="25" t="inlineStr">
+        <is>
+          <t>4. Add inside the Reels editor and mute your own audio — it won't get muted for copyright, and your reel lands on the song's page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="24" t="inlineStr">
+        <is>
+          <t>Sync trick</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="44" customHeight="1">
+      <c r="A23" s="25" t="inlineStr">
+        <is>
+          <t>If the track builds, put its swell on SHOT 3 — the orb finishing its blend. That's the moment the reel is selling. Land the peak on the wall-of-orbs reveal at the end.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A20:C20"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Reframe reel shots to honest launch framing
Replaces the retrospective "6 months of my life" opening — untrue for a
newly shipped app — with a launch framing: the grid reads as what a year
becomes, and the close states it shipped days ago and is live.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JLTsBRbD5LTCiR7DCK43kP
</commit_message>
<xml_diff>
--- a/memory-lane-reel.xlsx
+++ b/memory-lane-reel.xlsx
@@ -673,12 +673,12 @@
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>The full Lane — your wall of orbs, scrolling slowly</t>
+          <t>The full Lane / concept grid — what a year becomes</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>this is 6 months of my life</t>
+          <t>every day becomes one orb</t>
         </is>
       </c>
     </row>
@@ -888,7 +888,7 @@
       </c>
       <c r="H12" s="19" t="inlineStr">
         <is>
-          <t>i built this. it's live 👇</t>
+          <t>shipped it 3 days ago. it's live 👇</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rebuild reel shot list for a day-one app
The old shots asked for a filled Lane and a populated Journey screen, which
a three-day-old app cannot produce. Lead instead with the fill interaction,
which works on day one; show the real near-empty Lane honestly; and use the
full-year grid only as a labelled designed card, never a faked recording. A
Source column marks each shot as a real screen recording or a designed card.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JLTsBRbD5LTCiR7DCK43kP
</commit_message>
<xml_diff>
--- a/memory-lane-reel.xlsx
+++ b/memory-lane-reel.xlsx
@@ -572,37 +572,37 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="46" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Reel — Six months, one orb a day</t>
+          <t>Reel — one orb a day (day-1 honest cut)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>All 7 shots are SCREEN RECORDINGS of the live app. No camera, no tripod. Audio: a calm/aesthetic trending track added inside Instagram, not in your export.</t>
+          <t>Built for a brand-new app: leads with the FILL interaction (real, works today), shows your actual day-3 Lane honestly, and uses the full-year grid only as a DESIGNED CARD — never a faked screen recording. Audio added inside Instagram.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Blue cells are yours. Change a Duration and every timecode below re-syncs. Shot 3 (the orb filling) is the whole reel — hold on it.</t>
+          <t>'Source' says what each shot is. GREEN = real screen recording. BLUE = a designed graphic (reuse carousel 1 page 1). Blue Duration cells re-sync all timecodes.</t>
         </is>
       </c>
     </row>
@@ -614,7 +614,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Block</t>
+          <t>Source</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -639,7 +639,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>What you record</t>
+          <t>What you capture</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -648,86 +648,86 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="44" customHeight="1">
-      <c r="A6" s="4" t="n">
+    <row r="6" ht="46" customHeight="1">
+      <c r="A6" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>HERO</t>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>screen rec</t>
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="11">
         <f>D6+C6</f>
         <v/>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="11">
         <f>"0:"&amp;TEXT(D6,"00")&amp;" - 0:"&amp;TEXT(E6,"00")</f>
         <v/>
       </c>
-      <c r="G6" s="7" t="inlineStr">
-        <is>
-          <t>The full Lane / concept grid — what a year becomes</t>
-        </is>
-      </c>
-      <c r="H6" s="7" t="inlineStr">
-        <is>
-          <t>every day becomes one orb</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="44" customHeight="1">
-      <c r="A7" s="8" t="n">
+      <c r="G6" s="13" t="inlineStr">
+        <is>
+          <t>Extreme close on an EMPTY Today orb, then hold the emotions and let it blend LIVE</t>
+        </is>
+      </c>
+      <c r="H6" s="13" t="inlineStr">
+        <is>
+          <t>you don't write anything</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="46" customHeight="1">
+      <c r="A7" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>cut</t>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>screen rec</t>
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" s="8">
+        <v>2</v>
+      </c>
+      <c r="D7" s="11">
         <f>E6</f>
         <v/>
       </c>
-      <c r="E7" s="8">
+      <c r="E7" s="11">
         <f>D7+C7</f>
         <v/>
       </c>
-      <c r="F7" s="8">
+      <c r="F7" s="11">
         <f>"0:"&amp;TEXT(D7,"00")&amp;" - 0:"&amp;TEXT(E7,"00")</f>
         <v/>
       </c>
-      <c r="G7" s="10" t="inlineStr">
-        <is>
-          <t>Hard cut to one EMPTY Today orb</t>
-        </is>
-      </c>
-      <c r="H7" s="10" t="inlineStr">
-        <is>
-          <t>one orb a day</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="44" customHeight="1">
+      <c r="G7" s="13" t="inlineStr">
+        <is>
+          <t>The finished glazed sphere settles</t>
+        </is>
+      </c>
+      <c r="H7" s="13" t="inlineStr">
+        <is>
+          <t>you just hold how the day felt</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="46" customHeight="1">
       <c r="A8" s="11" t="n">
         <v>3</v>
       </c>
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>THE SHOT</t>
+          <t>screen rec</t>
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D8" s="11">
         <f>E7</f>
@@ -743,176 +743,160 @@
       </c>
       <c r="G8" s="13" t="inlineStr">
         <is>
-          <t>Hold-to-fill: press emotions, orb re-blends live. Real footage, not static.</t>
+          <t>It drops into your Lane — your REAL lane, a few orbs and blanks. This is day 3, show it honestly</t>
         </is>
       </c>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>(no text — let the blend speak)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="44" customHeight="1">
-      <c r="A9" s="14" t="n">
+          <t>one orb a day</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="46" customHeight="1">
+      <c r="A9" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="15" t="inlineStr">
-        <is>
-          <t>settle</t>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>designed card</t>
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D9" s="14">
+        <v>3</v>
+      </c>
+      <c r="D9" s="4">
         <f>E8</f>
         <v/>
       </c>
-      <c r="E9" s="14">
+      <c r="E9" s="4">
         <f>D9+C9</f>
         <v/>
       </c>
-      <c r="F9" s="14">
+      <c r="F9" s="4">
         <f>"0:"&amp;TEXT(D9,"00")&amp;" - 0:"&amp;TEXT(E9,"00")</f>
         <v/>
       </c>
-      <c r="G9" s="16" t="inlineStr">
-        <is>
-          <t>The finished glazed sphere settles</t>
-        </is>
-      </c>
-      <c r="H9" s="16" t="inlineStr">
-        <is>
-          <t>coloured by how the day felt</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="44" customHeight="1">
-      <c r="A10" s="14" t="n">
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>Cut to the full-year grid graphic (carousel 1 page 1). Clearly a designed card, not your screen</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>this is what a year becomes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="46" customHeight="1">
+      <c r="A10" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="15" t="inlineStr">
-        <is>
-          <t>drop</t>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>screen rec</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D10" s="14">
+      <c r="D10" s="11">
         <f>E9</f>
         <v/>
       </c>
-      <c r="E10" s="14">
+      <c r="E10" s="11">
         <f>D10+C10</f>
         <v/>
       </c>
-      <c r="F10" s="14">
+      <c r="F10" s="11">
         <f>"0:"&amp;TEXT(D10,"00")&amp;" - 0:"&amp;TEXT(E10,"00")</f>
         <v/>
       </c>
-      <c r="G10" s="16" t="inlineStr">
-        <is>
-          <t>It drops into the Lane beside the others</t>
-        </is>
-      </c>
-      <c r="H10" s="16" t="inlineStr">
-        <is>
-          <t>no writing. no prompt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="44" customHeight="1">
-      <c r="A11" s="11" t="n">
+      <c r="G10" s="13" t="inlineStr">
+        <is>
+          <t>Back in the app — open the emotion picker so the shared 100% pool is visible</t>
+        </is>
+      </c>
+      <c r="H10" s="13" t="inlineStr">
+        <is>
+          <t>a day only has 100% to give</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="46" customHeight="1">
+      <c r="A11" s="17" t="n">
         <v>6</v>
       </c>
-      <c r="B11" s="12" t="inlineStr">
-        <is>
-          <t>Journey</t>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>designed card</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D11" s="11">
+        <v>3</v>
+      </c>
+      <c r="D11" s="17">
         <f>E10</f>
         <v/>
       </c>
-      <c r="E11" s="11">
+      <c r="E11" s="17">
         <f>D11+C11</f>
         <v/>
       </c>
-      <c r="F11" s="11">
+      <c r="F11" s="17">
         <f>"0:"&amp;TEXT(D11,"00")&amp;" - 0:"&amp;TEXT(E11,"00")</f>
         <v/>
       </c>
-      <c r="G11" s="13" t="inlineStr">
-        <is>
-          <t>Journey screen — the standout days</t>
-        </is>
-      </c>
-      <c r="H11" s="13" t="inlineStr">
-        <is>
-          <t>the ones that mattered rise on their own</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="44" customHeight="1">
-      <c r="A12" s="17" t="n">
-        <v>7</v>
-      </c>
-      <c r="B12" s="18" t="inlineStr">
-        <is>
-          <t>CLOSE</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D12" s="17">
-        <f>E11</f>
-        <v/>
-      </c>
-      <c r="E12" s="17">
-        <f>D12+C12</f>
-        <v/>
-      </c>
-      <c r="F12" s="17">
-        <f>"0:"&amp;TEXT(D12,"00")&amp;" - 0:"&amp;TEXT(E12,"00")</f>
-        <v/>
-      </c>
-      <c r="G12" s="19" t="inlineStr">
-        <is>
-          <t>Back to the full wall, then your handle</t>
-        </is>
-      </c>
-      <c r="H12" s="19" t="inlineStr">
+      <c r="G11" s="19" t="inlineStr">
+        <is>
+          <t>App name / your handle over a soft orb</t>
+        </is>
+      </c>
+      <c r="H11" s="19" t="inlineStr">
         <is>
           <t>shipped it 3 days ago. it's live 👇</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="20" t="n"/>
-      <c r="B13" s="21" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="20" t="n"/>
+      <c r="B12" s="21" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C13" s="21">
-        <f>SUM(C6:C12)</f>
-        <v/>
-      </c>
-      <c r="D13" s="20" t="n"/>
-      <c r="E13" s="20" t="n"/>
-      <c r="F13" s="21">
-        <f>"0:"&amp;TEXT(SUM(C6:C12),"00")&amp;" total"</f>
-        <v/>
-      </c>
-      <c r="G13" s="20" t="n"/>
-      <c r="H13" s="20" t="n"/>
-    </row>
+      <c r="C12" s="21">
+        <f>SUM(C6:C11)</f>
+        <v/>
+      </c>
+      <c r="D12" s="20" t="n"/>
+      <c r="E12" s="20" t="n"/>
+      <c r="F12" s="21">
+        <f>"0:"&amp;TEXT(SUM(C6:C11),"00")&amp;" total"</f>
+        <v/>
+      </c>
+      <c r="G12" s="20" t="n"/>
+      <c r="H12" s="20" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="24" t="inlineStr">
+        <is>
+          <t>Why this cut</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="25" t="inlineStr">
+        <is>
+          <t>The fill interaction is the only genuinely magical thing that already works on day 1 — so it leads. Your real Lane is nearly empty, and that's fine: showing it honestly IS the build-in-public story. The gorgeous full-year wall still appears, but as a designed card labelled 'what a year becomes' — a vision, not a claim about your history. Nobody can call it fake because you never say it's yours.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16"/>
+    <row r="17"/>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A15:H17"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Rework reel as the build story: grind to gift
Restructures the reel around making the app rather than demoing it: real
code, PowerShell, streaming build logs, a real deployment error, late-night
commit timestamps, one tired human shot, the build finishing, then the app
working. Every shot is real footage the maker already has. Adds a source
guide per clip and retunes the music note toward a track that builds and
releases on the final reveal.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JLTsBRbD5LTCiR7DCK43kP
</commit_message>
<xml_diff>
--- a/memory-lane-reel.xlsx
+++ b/memory-lane-reel.xlsx
@@ -71,7 +71,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -113,8 +113,18 @@
         <fgColor rgb="00FBEFE9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3E9EC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FBF0DC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -136,11 +146,55 @@
         <color rgb="00C9CFD8"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00C9CFD8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C9CFD8"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C9CFD8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00C9CFD8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C9CFD8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C9CFD8"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C9CFD8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C9CFD8"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -207,6 +261,26 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -572,37 +646,37 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="48" customWidth="1" min="7" max="7"/>
-    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Reel — one orb a day (day-1 honest cut)</t>
+          <t>Reel — the build (grind → gift)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Built for a brand-new app: leads with the FILL interaction (real, works today), shows your actual day-3 Lane honestly, and uses the full-year grid only as a DESIGNED CARD — never a faked screen recording. Audio added inside Instagram.</t>
+          <t>The story of making it: your code, PowerShell, the build logs, the deployment errors, the sleepless nights — then the app. Every shot is REAL footage you already have. Nothing staged, nothing faked.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>'Source' says what each shot is. GREEN = real screen recording. BLUE = a designed graphic (reuse carousel 1 page 1). Blue Duration cells re-sync all timecodes.</t>
+          <t>Capture on your laptop (screen recordings) except shot 6, the one human shot. Blue Duration cells re-sync all timecodes. Music should BUILD and release on shot 8.</t>
         </is>
       </c>
     </row>
@@ -614,7 +688,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>Beat</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -639,7 +713,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>What you capture</t>
+          <t>What you capture (all real)</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -648,254 +722,483 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="46" customHeight="1">
-      <c r="A6" s="11" t="n">
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>screen rec</t>
+      <c r="B6" s="27" t="inlineStr">
+        <is>
+          <t>GRIND</t>
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="D6" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="11">
+      <c r="E6" s="26">
         <f>D6+C6</f>
         <v/>
       </c>
-      <c r="F6" s="11">
+      <c r="F6" s="26">
         <f>"0:"&amp;TEXT(D6,"00")&amp;" - 0:"&amp;TEXT(E6,"00")</f>
         <v/>
       </c>
-      <c r="G6" s="13" t="inlineStr">
-        <is>
-          <t>Extreme close on an EMPTY Today orb, then hold the emotions and let it blend LIVE</t>
-        </is>
-      </c>
-      <c r="H6" s="13" t="inlineStr">
-        <is>
-          <t>you don't write anything</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="46" customHeight="1">
-      <c r="A7" s="11" t="n">
+      <c r="G6" s="28" t="inlineStr">
+        <is>
+          <t>Your actual code — scroll the repo in VS Code, TypeScript / React Native flying past</t>
+        </is>
+      </c>
+      <c r="H6" s="28" t="inlineStr">
+        <is>
+          <t>3 days ago this didn't exist</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="12" t="inlineStr">
-        <is>
-          <t>screen rec</t>
+      <c r="B7" s="27" t="inlineStr">
+        <is>
+          <t>GRIND</t>
         </is>
       </c>
       <c r="C7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="11">
+      <c r="D7" s="26">
         <f>E6</f>
         <v/>
       </c>
-      <c r="E7" s="11">
+      <c r="E7" s="26">
         <f>D7+C7</f>
         <v/>
       </c>
-      <c r="F7" s="11">
+      <c r="F7" s="26">
         <f>"0:"&amp;TEXT(D7,"00")&amp;" - 0:"&amp;TEXT(E7,"00")</f>
         <v/>
       </c>
-      <c r="G7" s="13" t="inlineStr">
-        <is>
-          <t>The finished glazed sphere settles</t>
-        </is>
-      </c>
-      <c r="H7" s="13" t="inlineStr">
-        <is>
-          <t>you just hold how the day felt</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="46" customHeight="1">
-      <c r="A8" s="11" t="n">
+      <c r="G7" s="28" t="inlineStr">
+        <is>
+          <t>PowerShell running the build: type and run  eas build --platform android</t>
+        </is>
+      </c>
+      <c r="H7" s="28" t="inlineStr">
+        <is>
+          <t>so i built it</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t>screen rec</t>
+      <c r="B8" s="27" t="inlineStr">
+        <is>
+          <t>GRIND</t>
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D8" s="11">
+        <v>2</v>
+      </c>
+      <c r="D8" s="26">
         <f>E7</f>
         <v/>
       </c>
-      <c r="E8" s="11">
+      <c r="E8" s="26">
         <f>D8+C8</f>
         <v/>
       </c>
-      <c r="F8" s="11">
+      <c r="F8" s="26">
         <f>"0:"&amp;TEXT(D8,"00")&amp;" - 0:"&amp;TEXT(E8,"00")</f>
         <v/>
       </c>
-      <c r="G8" s="13" t="inlineStr">
-        <is>
-          <t>It drops into your Lane — your REAL lane, a few orbs and blanks. This is day 3, show it honestly</t>
-        </is>
-      </c>
-      <c r="H8" s="13" t="inlineStr">
-        <is>
-          <t>one orb a day</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="46" customHeight="1">
-      <c r="A9" s="4" t="n">
+      <c r="G8" s="28" t="inlineStr">
+        <is>
+          <t>The EAS build logs streaming — the real wall of build output</t>
+        </is>
+      </c>
+      <c r="H8" s="28" t="inlineStr">
+        <is>
+          <t>every line of it myself</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>designed card</t>
+      <c r="B9" s="27" t="inlineStr">
+        <is>
+          <t>GRIND</t>
         </is>
       </c>
       <c r="C9" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="26">
         <f>E8</f>
         <v/>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="26">
         <f>D9+C9</f>
         <v/>
       </c>
-      <c r="F9" s="4">
+      <c r="F9" s="26">
         <f>"0:"&amp;TEXT(D9,"00")&amp;" - 0:"&amp;TEXT(E9,"00")</f>
         <v/>
       </c>
-      <c r="G9" s="7" t="inlineStr">
-        <is>
-          <t>Cut to the full-year grid graphic (carousel 1 page 1). Clearly a designed card, not your screen</t>
-        </is>
-      </c>
-      <c r="H9" s="7" t="inlineStr">
-        <is>
-          <t>this is what a year becomes</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="46" customHeight="1">
-      <c r="A10" s="11" t="n">
+      <c r="G9" s="28" t="inlineStr">
+        <is>
+          <t>The RED. A real deployment error / failed build. Hold on the red text</t>
+        </is>
+      </c>
+      <c r="H9" s="28" t="inlineStr">
+        <is>
+          <t>it broke. a lot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="12" t="inlineStr">
-        <is>
-          <t>screen rec</t>
+      <c r="B10" s="27" t="inlineStr">
+        <is>
+          <t>GRIND</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D10" s="11">
+      <c r="D10" s="26">
         <f>E9</f>
         <v/>
       </c>
-      <c r="E10" s="11">
+      <c r="E10" s="26">
         <f>D10+C10</f>
         <v/>
       </c>
-      <c r="F10" s="11">
+      <c r="F10" s="26">
         <f>"0:"&amp;TEXT(D10,"00")&amp;" - 0:"&amp;TEXT(E10,"00")</f>
         <v/>
       </c>
-      <c r="G10" s="13" t="inlineStr">
-        <is>
-          <t>Back in the app — open the emotion picker so the shared 100% pool is visible</t>
-        </is>
-      </c>
-      <c r="H10" s="13" t="inlineStr">
-        <is>
-          <t>a day only has 100% to give</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="46" customHeight="1">
-      <c r="A11" s="17" t="n">
+      <c r="G10" s="28" t="inlineStr">
+        <is>
+          <t>git log with your real late-night timestamps — 2am, 3am commits</t>
+        </is>
+      </c>
+      <c r="H10" s="28" t="inlineStr">
+        <is>
+          <t>2am. 3am. again.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="B11" s="18" t="inlineStr">
-        <is>
-          <t>designed card</t>
+      <c r="B11" s="27" t="inlineStr">
+        <is>
+          <t>HUMAN</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D11" s="17">
+        <v>2</v>
+      </c>
+      <c r="D11" s="26">
         <f>E10</f>
         <v/>
       </c>
-      <c r="E11" s="17">
+      <c r="E11" s="26">
         <f>D11+C11</f>
         <v/>
       </c>
-      <c r="F11" s="17">
+      <c r="F11" s="26">
         <f>"0:"&amp;TEXT(D11,"00")&amp;" - 0:"&amp;TEXT(E11,"00")</f>
         <v/>
       </c>
-      <c r="G11" s="19" t="inlineStr">
-        <is>
-          <t>App name / your handle over a soft orb</t>
-        </is>
-      </c>
-      <c r="H11" s="19" t="inlineStr">
-        <is>
-          <t>shipped it 3 days ago. it's live 👇</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="20" t="n"/>
-      <c r="B12" s="21" t="inlineStr">
+      <c r="G11" s="28" t="inlineStr">
+        <is>
+          <t>ONE camera shot: you at the desk, dark room, laptop glow, head down. Tired</t>
+        </is>
+      </c>
+      <c r="H11" s="28" t="inlineStr">
+        <is>
+          <t>i almost gave up on it</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="29" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="30" t="inlineStr">
+        <is>
+          <t>TURN</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" s="29">
+        <f>E11</f>
+        <v/>
+      </c>
+      <c r="E12" s="29">
+        <f>D12+C12</f>
+        <v/>
+      </c>
+      <c r="F12" s="29">
+        <f>"0:"&amp;TEXT(D12,"00")&amp;" - 0:"&amp;TEXT(E12,"00")</f>
+        <v/>
+      </c>
+      <c r="G12" s="31" t="inlineStr">
+        <is>
+          <t>Build succeeded — the QR code / 'Build finished' / the install link appears</t>
+        </is>
+      </c>
+      <c r="H12" s="31" t="inlineStr">
+        <is>
+          <t>then it shipped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>GIFT</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D13" s="11">
+        <f>E12</f>
+        <v/>
+      </c>
+      <c r="E13" s="11">
+        <f>D13+C13</f>
+        <v/>
+      </c>
+      <c r="F13" s="11">
+        <f>"0:"&amp;TEXT(D13,"00")&amp;" - 0:"&amp;TEXT(E13,"00")</f>
+        <v/>
+      </c>
+      <c r="G13" s="13" t="inlineStr">
+        <is>
+          <t>The app opens. Fill an orb, watch it blend. It works. Hold on the finished sphere</t>
+        </is>
+      </c>
+      <c r="H13" s="13" t="inlineStr">
+        <is>
+          <t>and now it's real. it's live 👇</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="20" t="n"/>
+      <c r="B14" s="21" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C12" s="21">
-        <f>SUM(C6:C11)</f>
-        <v/>
-      </c>
-      <c r="D12" s="20" t="n"/>
-      <c r="E12" s="20" t="n"/>
-      <c r="F12" s="21">
-        <f>"0:"&amp;TEXT(SUM(C6:C11),"00")&amp;" total"</f>
-        <v/>
-      </c>
-      <c r="G12" s="20" t="n"/>
-      <c r="H12" s="20" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="24" t="inlineStr">
-        <is>
-          <t>Why this cut</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="25" t="inlineStr">
-        <is>
-          <t>The fill interaction is the only genuinely magical thing that already works on day 1 — so it leads. Your real Lane is nearly empty, and that's fine: showing it honestly IS the build-in-public story. The gorgeous full-year wall still appears, but as a designed card labelled 'what a year becomes' — a vision, not a claim about your history. Nobody can call it fake because you never say it's yours.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16"/>
-    <row r="17"/>
+      <c r="C14" s="21">
+        <f>SUM(C6:C13)</f>
+        <v/>
+      </c>
+      <c r="D14" s="20" t="n"/>
+      <c r="E14" s="20" t="n"/>
+      <c r="F14" s="21">
+        <f>"0:"&amp;TEXT(SUM(C6:C13),"00")&amp;" total"</f>
+        <v/>
+      </c>
+      <c r="G14" s="20" t="n"/>
+      <c r="H14" s="20" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="24" t="inlineStr">
+        <is>
+          <t>The shape</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="25" t="inlineStr">
+        <is>
+          <t>Shots 1-6 are the GRIND — fast, tense, cut hard on the beat. They get faster and messier toward the red error and the 3am commits. Shot 7 is the TURN, one breath. Shot 8 is the GIFT — let it breathe, hold on the orb, this is the whole reel paying off. Grind = tight cuts, gift = the longest shot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="21">
+      <c r="A21" s="24" t="inlineStr">
+        <is>
+          <t>Where each real clip comes from</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="23" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="B22" s="22" t="inlineStr">
+        <is>
+          <t>Open the repo in VS Code, screen-record a slow scroll through a .tsx file.</t>
+        </is>
+      </c>
+      <c r="C22" s="32" t="n"/>
+      <c r="D22" s="32" t="n"/>
+      <c r="E22" s="32" t="n"/>
+      <c r="F22" s="32" t="n"/>
+      <c r="G22" s="32" t="n"/>
+      <c r="H22" s="33" t="n"/>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="23" t="inlineStr">
+        <is>
+          <t>PowerShell</t>
+        </is>
+      </c>
+      <c r="B23" s="22" t="inlineStr">
+        <is>
+          <t>Screen-record the terminal as you run the eas build command.</t>
+        </is>
+      </c>
+      <c r="C23" s="32" t="n"/>
+      <c r="D23" s="32" t="n"/>
+      <c r="E23" s="32" t="n"/>
+      <c r="F23" s="32" t="n"/>
+      <c r="G23" s="32" t="n"/>
+      <c r="H23" s="33" t="n"/>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="23" t="inlineStr">
+        <is>
+          <t>Build logs</t>
+        </is>
+      </c>
+      <c r="B24" s="22" t="inlineStr">
+        <is>
+          <t>The EAS build page in your browser, logs streaming — screen-record it.</t>
+        </is>
+      </c>
+      <c r="C24" s="32" t="n"/>
+      <c r="D24" s="32" t="n"/>
+      <c r="E24" s="32" t="n"/>
+      <c r="F24" s="32" t="n"/>
+      <c r="G24" s="32" t="n"/>
+      <c r="H24" s="33" t="n"/>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="23" t="inlineStr">
+        <is>
+          <t>The red error</t>
+        </is>
+      </c>
+      <c r="B25" s="22" t="inlineStr">
+        <is>
+          <t>A real failed build / deployment error. If you have a screenshot, use it; else re-trigger one.</t>
+        </is>
+      </c>
+      <c r="C25" s="32" t="n"/>
+      <c r="D25" s="32" t="n"/>
+      <c r="E25" s="32" t="n"/>
+      <c r="F25" s="32" t="n"/>
+      <c r="G25" s="32" t="n"/>
+      <c r="H25" s="33" t="n"/>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="23" t="inlineStr">
+        <is>
+          <t>Sleepless nights</t>
+        </is>
+      </c>
+      <c r="B26" s="22" t="inlineStr">
+        <is>
+          <t>git log --oneline --date=format:'%H:%M' — your real late commit times. Or a screenshot of a 3am commit.</t>
+        </is>
+      </c>
+      <c r="C26" s="32" t="n"/>
+      <c r="D26" s="32" t="n"/>
+      <c r="E26" s="32" t="n"/>
+      <c r="F26" s="32" t="n"/>
+      <c r="G26" s="32" t="n"/>
+      <c r="H26" s="33" t="n"/>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="23" t="inlineStr">
+        <is>
+          <t>The human shot</t>
+        </is>
+      </c>
+      <c r="B27" s="22" t="inlineStr">
+        <is>
+          <t>Phone on books, dark room, laptop light on your face, head in hand. 6 seconds, one take.</t>
+        </is>
+      </c>
+      <c r="C27" s="32" t="n"/>
+      <c r="D27" s="32" t="n"/>
+      <c r="E27" s="32" t="n"/>
+      <c r="F27" s="32" t="n"/>
+      <c r="G27" s="32" t="n"/>
+      <c r="H27" s="33" t="n"/>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="23" t="inlineStr">
+        <is>
+          <t>The turn</t>
+        </is>
+      </c>
+      <c r="B28" s="22" t="inlineStr">
+        <is>
+          <t>Your QR code / install link / 'Build finished 🎉' — you already have this.</t>
+        </is>
+      </c>
+      <c r="C28" s="32" t="n"/>
+      <c r="D28" s="32" t="n"/>
+      <c r="E28" s="32" t="n"/>
+      <c r="F28" s="32" t="n"/>
+      <c r="G28" s="32" t="n"/>
+      <c r="H28" s="33" t="n"/>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="23" t="inlineStr">
+        <is>
+          <t>The gift</t>
+        </is>
+      </c>
+      <c r="B29" s="22" t="inlineStr">
+        <is>
+          <t>Screen-record the app: open it, fill an orb, the blend. The real magic.</t>
+        </is>
+      </c>
+      <c r="C29" s="32" t="n"/>
+      <c r="D29" s="32" t="n"/>
+      <c r="E29" s="32" t="n"/>
+      <c r="F29" s="32" t="n"/>
+      <c r="G29" s="32" t="n"/>
+      <c r="H29" s="33" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A15:H17"/>
+  <mergeCells count="9">
+    <mergeCell ref="B22:H22"/>
+    <mergeCell ref="A17:H19"/>
+    <mergeCell ref="B26:H26"/>
+    <mergeCell ref="B27:H27"/>
+    <mergeCell ref="B24:H24"/>
+    <mergeCell ref="B29:H29"/>
+    <mergeCell ref="B25:H25"/>
+    <mergeCell ref="B28:H28"/>
+    <mergeCell ref="B23:H23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1413,7 +1716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1430,7 +1733,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Calm, warm, slightly nostalgic, building gently. Softer than a launch hype edit. Add it INSIDE Instagram, mute your export.</t>
+          <t>This reel is a BUILD: tense grind, then release on the app reveal. The track must build and peak on shot 8. Add it inside Instagram, mute your export.</t>
         </is>
       </c>
     </row>
@@ -1617,12 +1920,29 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="24" t="inlineStr">
+        <is>
+          <t>For THIS reel specifically</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="25" t="inlineStr">
+        <is>
+          <t>The calm tracks above suit a gentle product reel. This grind-to-gift version wants a track that BUILDS — quiet/tense under the code and errors, then swells or drops exactly on shot 8 when the app works. Search: 'emotional build', 'cinematic build up', or a song with a clear drop. Put the drop on the orb reveal. That single sync is what makes people feel it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27"/>
+    <row r="28"/>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="A19:C19"/>
     <mergeCell ref="A23:C23"/>
     <mergeCell ref="A17:C17"/>
     <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A26:C28"/>
     <mergeCell ref="A20:C20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Extend the build reel to a ~30s story arc
Lengthens the grind-to-gift reel from 8 to 12 shots: a clearer start from
nothing, two distinct error beats, the install-on-a-real-phone moment, and a
longer payoff on the working app. Adds pacing notes — grind accelerates,
gift breathes.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JLTsBRbD5LTCiR7DCK43kP
</commit_message>
<xml_diff>
--- a/memory-lane-reel.xlsx
+++ b/memory-lane-reel.xlsx
@@ -646,7 +646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -662,21 +662,21 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Reel — the build (grind → gift)</t>
+          <t>Reel — the build (grind → gift) · ~26s</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>The story of making it: your code, PowerShell, the build logs, the deployment errors, the sleepless nights — then the app. Every shot is REAL footage you already have. Nothing staged, nothing faked.</t>
+          <t>The longer cut. Same story, more room: the build, the tools fighting back, the errors, the nights, the near-quit, the ship, and the app. Every shot is REAL footage you already have.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Capture on your laptop (screen recordings) except shot 6, the one human shot. Blue Duration cells re-sync all timecodes. Music should BUILD and release on shot 8.</t>
+          <t>Grind gets faster toward the bottom; the gift breathes. Blue Duration cells re-sync every timecode. Music must build and release on the final orb.</t>
         </is>
       </c>
     </row>
@@ -722,7 +722,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="48" customHeight="1">
+    <row r="6" ht="46" customHeight="1">
       <c r="A6" s="26" t="n">
         <v>1</v>
       </c>
@@ -747,16 +747,16 @@
       </c>
       <c r="G6" s="28" t="inlineStr">
         <is>
-          <t>Your actual code — scroll the repo in VS Code, TypeScript / React Native flying past</t>
+          <t>An empty VS Code project / a blank folder. Then the first file appears</t>
         </is>
       </c>
       <c r="H6" s="28" t="inlineStr">
         <is>
-          <t>3 days ago this didn't exist</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="48" customHeight="1">
+          <t>3 days ago this was nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="46" customHeight="1">
       <c r="A7" s="26" t="n">
         <v>2</v>
       </c>
@@ -782,16 +782,16 @@
       </c>
       <c r="G7" s="28" t="inlineStr">
         <is>
-          <t>PowerShell running the build: type and run  eas build --platform android</t>
+          <t>Your code — scroll a .tsx file, TypeScript / React Native flying past</t>
         </is>
       </c>
       <c r="H7" s="28" t="inlineStr">
         <is>
-          <t>so i built it</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="48" customHeight="1">
+          <t>so i started building</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="46" customHeight="1">
       <c r="A8" s="26" t="n">
         <v>3</v>
       </c>
@@ -817,16 +817,16 @@
       </c>
       <c r="G8" s="28" t="inlineStr">
         <is>
-          <t>The EAS build logs streaming — the real wall of build output</t>
+          <t>PowerShell: type and run  eas build --platform android</t>
         </is>
       </c>
       <c r="H8" s="28" t="inlineStr">
         <is>
-          <t>every line of it myself</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="48" customHeight="1">
+          <t>one command to ship it</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="46" customHeight="1">
       <c r="A9" s="26" t="n">
         <v>4</v>
       </c>
@@ -852,16 +852,16 @@
       </c>
       <c r="G9" s="28" t="inlineStr">
         <is>
-          <t>The RED. A real deployment error / failed build. Hold on the red text</t>
+          <t>The EAS build logs streaming — the real wall of output</t>
         </is>
       </c>
       <c r="H9" s="28" t="inlineStr">
         <is>
-          <t>it broke. a lot.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="48" customHeight="1">
+          <t>or so i thought</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="46" customHeight="1">
       <c r="A10" s="26" t="n">
         <v>5</v>
       </c>
@@ -871,7 +871,7 @@
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D10" s="26">
         <f>E9</f>
@@ -887,22 +887,22 @@
       </c>
       <c r="G10" s="28" t="inlineStr">
         <is>
-          <t>git log with your real late-night timestamps — 2am, 3am commits</t>
+          <t>The RED. A real deployment error / failed build. Hold on it</t>
         </is>
       </c>
       <c r="H10" s="28" t="inlineStr">
         <is>
-          <t>2am. 3am. again.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="48" customHeight="1">
+          <t>it broke.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="46" customHeight="1">
       <c r="A11" s="26" t="n">
         <v>6</v>
       </c>
       <c r="B11" s="27" t="inlineStr">
         <is>
-          <t>HUMAN</t>
+          <t>GRIND</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
@@ -922,283 +922,264 @@
       </c>
       <c r="G11" s="28" t="inlineStr">
         <is>
-          <t>ONE camera shot: you at the desk, dark room, laptop glow, head down. Tired</t>
+          <t>A different error — config / dependency / gradle. More red</t>
         </is>
       </c>
       <c r="H11" s="28" t="inlineStr">
         <is>
-          <t>i almost gave up on it</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="48" customHeight="1">
-      <c r="A12" s="29" t="n">
+          <t>and broke again.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="46" customHeight="1">
+      <c r="A12" s="26" t="n">
         <v>7</v>
       </c>
-      <c r="B12" s="30" t="inlineStr">
-        <is>
-          <t>TURN</t>
+      <c r="B12" s="27" t="inlineStr">
+        <is>
+          <t>GRIND</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="29">
+      <c r="D12" s="26">
         <f>E11</f>
         <v/>
       </c>
-      <c r="E12" s="29">
+      <c r="E12" s="26">
         <f>D12+C12</f>
         <v/>
       </c>
-      <c r="F12" s="29">
+      <c r="F12" s="26">
         <f>"0:"&amp;TEXT(D12,"00")&amp;" - 0:"&amp;TEXT(E12,"00")</f>
         <v/>
       </c>
-      <c r="G12" s="31" t="inlineStr">
-        <is>
-          <t>Build succeeded — the QR code / 'Build finished' / the install link appears</t>
-        </is>
-      </c>
-      <c r="H12" s="31" t="inlineStr">
-        <is>
-          <t>then it shipped.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="48" customHeight="1">
-      <c r="A13" s="11" t="n">
+      <c r="G12" s="28" t="inlineStr">
+        <is>
+          <t>git log with your real late timestamps — 2am, 3am commits</t>
+        </is>
+      </c>
+      <c r="H12" s="28" t="inlineStr">
+        <is>
+          <t>2am. 3am. 2am.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="46" customHeight="1">
+      <c r="A13" s="26" t="n">
         <v>8</v>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B13" s="27" t="inlineStr">
+        <is>
+          <t>HUMAN</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D13" s="26">
+        <f>E12</f>
+        <v/>
+      </c>
+      <c r="E13" s="26">
+        <f>D13+C13</f>
+        <v/>
+      </c>
+      <c r="F13" s="26">
+        <f>"0:"&amp;TEXT(D13,"00")&amp;" - 0:"&amp;TEXT(E13,"00")</f>
+        <v/>
+      </c>
+      <c r="G13" s="28" t="inlineStr">
+        <is>
+          <t>ONE camera shot: you at the desk, dark room, laptop glow, head in hand</t>
+        </is>
+      </c>
+      <c r="H13" s="28" t="inlineStr">
+        <is>
+          <t>i almost deleted the whole thing</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="46" customHeight="1">
+      <c r="A14" s="29" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" s="30" t="inlineStr">
+        <is>
+          <t>TURN</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" s="29">
+        <f>E13</f>
+        <v/>
+      </c>
+      <c r="E14" s="29">
+        <f>D14+C14</f>
+        <v/>
+      </c>
+      <c r="F14" s="29">
+        <f>"0:"&amp;TEXT(D14,"00")&amp;" - 0:"&amp;TEXT(E14,"00")</f>
+        <v/>
+      </c>
+      <c r="G14" s="31" t="inlineStr">
+        <is>
+          <t>Build SUCCEEDED — 'Build finished', the QR code, the install link</t>
+        </is>
+      </c>
+      <c r="H14" s="31" t="inlineStr">
+        <is>
+          <t>then — it built.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="46" customHeight="1">
+      <c r="A15" s="29" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" s="30" t="inlineStr">
+        <is>
+          <t>TURN</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" s="29">
+        <f>E14</f>
+        <v/>
+      </c>
+      <c r="E15" s="29">
+        <f>D15+C15</f>
+        <v/>
+      </c>
+      <c r="F15" s="29">
+        <f>"0:"&amp;TEXT(D15,"00")&amp;" - 0:"&amp;TEXT(E15,"00")</f>
+        <v/>
+      </c>
+      <c r="G15" s="31" t="inlineStr">
+        <is>
+          <t>The app installing on your real phone / the icon appearing on the home screen</t>
+        </is>
+      </c>
+      <c r="H15" s="31" t="inlineStr">
+        <is>
+          <t>it installed on a real phone</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="46" customHeight="1">
+      <c r="A16" s="11" t="n">
+        <v>11</v>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>GIFT</t>
         </is>
       </c>
-      <c r="C13" s="6" t="n">
+      <c r="C16" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="D13" s="11">
-        <f>E12</f>
-        <v/>
-      </c>
-      <c r="E13" s="11">
-        <f>D13+C13</f>
-        <v/>
-      </c>
-      <c r="F13" s="11">
-        <f>"0:"&amp;TEXT(D13,"00")&amp;" - 0:"&amp;TEXT(E13,"00")</f>
-        <v/>
-      </c>
-      <c r="G13" s="13" t="inlineStr">
-        <is>
-          <t>The app opens. Fill an orb, watch it blend. It works. Hold on the finished sphere</t>
-        </is>
-      </c>
-      <c r="H13" s="13" t="inlineStr">
-        <is>
-          <t>and now it's real. it's live 👇</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="20" t="n"/>
-      <c r="B14" s="21" t="inlineStr">
+      <c r="D16" s="11">
+        <f>E15</f>
+        <v/>
+      </c>
+      <c r="E16" s="11">
+        <f>D16+C16</f>
+        <v/>
+      </c>
+      <c r="F16" s="11">
+        <f>"0:"&amp;TEXT(D16,"00")&amp;" - 0:"&amp;TEXT(E16,"00")</f>
+        <v/>
+      </c>
+      <c r="G16" s="13" t="inlineStr">
+        <is>
+          <t>Open the app. Fill an orb, watch it blend live. It works. Hold on the sphere</t>
+        </is>
+      </c>
+      <c r="H16" s="13" t="inlineStr">
+        <is>
+          <t>and it actually works</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="46" customHeight="1">
+      <c r="A17" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>GIFT</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D17" s="11">
+        <f>E16</f>
+        <v/>
+      </c>
+      <c r="E17" s="11">
+        <f>D17+C17</f>
+        <v/>
+      </c>
+      <c r="F17" s="11">
+        <f>"0:"&amp;TEXT(D17,"00")&amp;" - 0:"&amp;TEXT(E17,"00")</f>
+        <v/>
+      </c>
+      <c r="G17" s="13" t="inlineStr">
+        <is>
+          <t>Your handle / the install link over a soft orb</t>
+        </is>
+      </c>
+      <c r="H17" s="13" t="inlineStr">
+        <is>
+          <t>i built this. it's live 👇</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="20" t="n"/>
+      <c r="B18" s="21" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C14" s="21">
-        <f>SUM(C6:C13)</f>
-        <v/>
-      </c>
-      <c r="D14" s="20" t="n"/>
-      <c r="E14" s="20" t="n"/>
-      <c r="F14" s="21">
-        <f>"0:"&amp;TEXT(SUM(C6:C13),"00")&amp;" total"</f>
-        <v/>
-      </c>
-      <c r="G14" s="20" t="n"/>
-      <c r="H14" s="20" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="24" t="inlineStr">
-        <is>
-          <t>The shape</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="25" t="inlineStr">
-        <is>
-          <t>Shots 1-6 are the GRIND — fast, tense, cut hard on the beat. They get faster and messier toward the red error and the 3am commits. Shot 7 is the TURN, one breath. Shot 8 is the GIFT — let it breathe, hold on the orb, this is the whole reel paying off. Grind = tight cuts, gift = the longest shot.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18"/>
-    <row r="19"/>
+      <c r="C18" s="21">
+        <f>SUM(C6:C17)</f>
+        <v/>
+      </c>
+      <c r="D18" s="20" t="n"/>
+      <c r="E18" s="20" t="n"/>
+      <c r="F18" s="21">
+        <f>"0:"&amp;TEXT(SUM(C6:C17),"00")&amp;" total"</f>
+        <v/>
+      </c>
+      <c r="G18" s="20" t="n"/>
+      <c r="H18" s="20" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="24" t="inlineStr">
+        <is>
+          <t>Pacing</t>
+        </is>
+      </c>
+    </row>
     <row r="21">
-      <c r="A21" s="24" t="inlineStr">
-        <is>
-          <t>Where each real clip comes from</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="23" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-      <c r="B22" s="22" t="inlineStr">
-        <is>
-          <t>Open the repo in VS Code, screen-record a slow scroll through a .tsx file.</t>
-        </is>
-      </c>
-      <c r="C22" s="32" t="n"/>
-      <c r="D22" s="32" t="n"/>
-      <c r="E22" s="32" t="n"/>
-      <c r="F22" s="32" t="n"/>
-      <c r="G22" s="32" t="n"/>
-      <c r="H22" s="33" t="n"/>
-    </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="23" t="inlineStr">
-        <is>
-          <t>PowerShell</t>
-        </is>
-      </c>
-      <c r="B23" s="22" t="inlineStr">
-        <is>
-          <t>Screen-record the terminal as you run the eas build command.</t>
-        </is>
-      </c>
-      <c r="C23" s="32" t="n"/>
-      <c r="D23" s="32" t="n"/>
-      <c r="E23" s="32" t="n"/>
-      <c r="F23" s="32" t="n"/>
-      <c r="G23" s="32" t="n"/>
-      <c r="H23" s="33" t="n"/>
-    </row>
-    <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="23" t="inlineStr">
-        <is>
-          <t>Build logs</t>
-        </is>
-      </c>
-      <c r="B24" s="22" t="inlineStr">
-        <is>
-          <t>The EAS build page in your browser, logs streaming — screen-record it.</t>
-        </is>
-      </c>
-      <c r="C24" s="32" t="n"/>
-      <c r="D24" s="32" t="n"/>
-      <c r="E24" s="32" t="n"/>
-      <c r="F24" s="32" t="n"/>
-      <c r="G24" s="32" t="n"/>
-      <c r="H24" s="33" t="n"/>
-    </row>
-    <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="23" t="inlineStr">
-        <is>
-          <t>The red error</t>
-        </is>
-      </c>
-      <c r="B25" s="22" t="inlineStr">
-        <is>
-          <t>A real failed build / deployment error. If you have a screenshot, use it; else re-trigger one.</t>
-        </is>
-      </c>
-      <c r="C25" s="32" t="n"/>
-      <c r="D25" s="32" t="n"/>
-      <c r="E25" s="32" t="n"/>
-      <c r="F25" s="32" t="n"/>
-      <c r="G25" s="32" t="n"/>
-      <c r="H25" s="33" t="n"/>
-    </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="23" t="inlineStr">
-        <is>
-          <t>Sleepless nights</t>
-        </is>
-      </c>
-      <c r="B26" s="22" t="inlineStr">
-        <is>
-          <t>git log --oneline --date=format:'%H:%M' — your real late commit times. Or a screenshot of a 3am commit.</t>
-        </is>
-      </c>
-      <c r="C26" s="32" t="n"/>
-      <c r="D26" s="32" t="n"/>
-      <c r="E26" s="32" t="n"/>
-      <c r="F26" s="32" t="n"/>
-      <c r="G26" s="32" t="n"/>
-      <c r="H26" s="33" t="n"/>
-    </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="23" t="inlineStr">
-        <is>
-          <t>The human shot</t>
-        </is>
-      </c>
-      <c r="B27" s="22" t="inlineStr">
-        <is>
-          <t>Phone on books, dark room, laptop light on your face, head in hand. 6 seconds, one take.</t>
-        </is>
-      </c>
-      <c r="C27" s="32" t="n"/>
-      <c r="D27" s="32" t="n"/>
-      <c r="E27" s="32" t="n"/>
-      <c r="F27" s="32" t="n"/>
-      <c r="G27" s="32" t="n"/>
-      <c r="H27" s="33" t="n"/>
-    </row>
-    <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="23" t="inlineStr">
-        <is>
-          <t>The turn</t>
-        </is>
-      </c>
-      <c r="B28" s="22" t="inlineStr">
-        <is>
-          <t>Your QR code / install link / 'Build finished 🎉' — you already have this.</t>
-        </is>
-      </c>
-      <c r="C28" s="32" t="n"/>
-      <c r="D28" s="32" t="n"/>
-      <c r="E28" s="32" t="n"/>
-      <c r="F28" s="32" t="n"/>
-      <c r="G28" s="32" t="n"/>
-      <c r="H28" s="33" t="n"/>
-    </row>
-    <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="23" t="inlineStr">
-        <is>
-          <t>The gift</t>
-        </is>
-      </c>
-      <c r="B29" s="22" t="inlineStr">
-        <is>
-          <t>Screen-record the app: open it, fill an orb, the blend. The real magic.</t>
-        </is>
-      </c>
-      <c r="C29" s="32" t="n"/>
-      <c r="D29" s="32" t="n"/>
-      <c r="E29" s="32" t="n"/>
-      <c r="F29" s="32" t="n"/>
-      <c r="G29" s="32" t="n"/>
-      <c r="H29" s="33" t="n"/>
-    </row>
+      <c r="A21" s="25" t="inlineStr">
+        <is>
+          <t>Shots 1-7 are the GRIND — they should speed UP as they go: 3s at the top, down to 2s by the 3am commits, cutting harder and messier toward the red. Shot 8 (the human beat) is the bottom — hold it, let it be still. Shots 9-10 are the TURN, the exhale. Shots 11-12 are the GIFT — the longest, calmest shots in the reel. The whole thing is tension tightening, then release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23"/>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="B22:H22"/>
-    <mergeCell ref="A17:H19"/>
-    <mergeCell ref="B26:H26"/>
-    <mergeCell ref="B27:H27"/>
-    <mergeCell ref="B24:H24"/>
-    <mergeCell ref="B29:H29"/>
-    <mergeCell ref="B25:H25"/>
-    <mergeCell ref="B28:H28"/>
-    <mergeCell ref="B23:H23"/>
+  <mergeCells count="1">
+    <mergeCell ref="A21:H23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fully direct the reel's desk shot for a tripod
Replaces the stack-of-books references with tripod placement, and expands
the desk-shot sheet into full direction: exact tripod position, lighting
(laptop-only, bright screen), wardrobe, body language, the 8-second action,
and a pre-roll checklist.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JLTsBRbD5LTCiR7DCK43kP
</commit_message>
<xml_diff>
--- a/memory-lane-reel.xlsx
+++ b/memory-lane-reel.xlsx
@@ -135,7 +135,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -157,11 +157,44 @@
         <color rgb="00C9CFD8"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00C9CFD8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C9CFD8"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C9CFD8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C9CFD8"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C9CFD8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C9CFD8"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -248,6 +281,10 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2180,7 +2217,7 @@
       </c>
       <c r="B41" s="9" t="inlineStr">
         <is>
-          <t>Phone on a stack of books, dark room, only the laptop lighting your face. Sit slumped, head in hand, still. One 8s take, use the calmest.</t>
+          <t>Tripod behind you, low, dark room, only the laptop lighting your face. Sit slumped, head in hand, still. One 8s take, use the calmest.</t>
         </is>
       </c>
     </row>
@@ -2788,133 +2825,477 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:B50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="84" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The Desk Shot — shot 8, the only thing you film</t>
+          <t>The Desk Shot — shot 8, fully directed</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>The emotional bottom of the reel. Dark, still, tired. One setup, one take you keep.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Element</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
+          <t>The one shot you film. The emotional bottom of the reel: dark, tired, still. Everything below is set before you roll.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>1 · TRIPOD PLACEMENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Setting</t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Camera</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>Your phone, on a stack of books behind you / to your side. Vertical 9:16.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="32" customHeight="1">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="38" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Where</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Room dark. ONLY the laptop screen on your face. No lamp.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="32" customHeight="1">
+          <t>BEHIND your chair, slightly to one side (in the walkway, not in front of the desk). It sees your head/shoulder and the laptop glowing in front of you.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="38" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Framing</t>
+          <t>Height</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Mid shot — you, the laptop glow, the dark around you. Leave the top third for text.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="32" customHeight="1">
+          <t>Chest-to-eye height, ~1.2–1.5m. Level with your head — NOT high looking down (that reads like a webcam).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="38" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>You</t>
+          <t>Distance</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Slumped, head in one hand, still. Not acting tired — just be still and let the dark do it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="32" customHeight="1">
+          <t>1.5–2m back. A mid shot: you, the laptop glow, dark around you. Not a close-up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="38" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Duration</t>
+          <t>Angle</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Record 8 seconds, use ~3. Do 2-3 takes; the stillest one wins.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="32" customHeight="1">
+          <t>Level or a hair down. Tilt so the TOP THIRD of frame is dark — that's where the text sits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="38" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Lock focus/exposure</t>
+          <t>Orientation</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Tap-and-hold on your face until it locks, so it doesn't hunt in the dark.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="32" customHeight="1">
+          <t>VERTICAL 9:16. Check the mount grips portrait, not just landscape.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="38" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Do Not Disturb</t>
+          <t>Lock it</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>On. And no notification light on the laptop.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="44" customHeight="1">
-      <c r="A13" s="23" t="inlineStr">
-        <is>
-          <t>Why it matters: shots 1-7 are all screen. This is the one moment a face appears — the human low point before the turn. It's what makes people feel the story instead of just watching a build. Hold it a beat longer than feels comfortable.</t>
-        </is>
-      </c>
+          <t>Legs locked, mount tight. Set it once, then don't touch it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>2 · LIGHTING</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="40" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>The only light</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Your LAPTOP SCREEN. Turn everything else off — overhead, lamp, phone torch. Full dark except the screen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Put a bright screen up</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Open something white/bright (a doc, the EAS logs, VS Code light theme) so the screen actually lights your face. A dark terminal won't.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="40" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Screen brightness</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>All the way up, and turn OFF auto-brightness so it doesn't dim mid-take.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="40" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>The look you want</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Screen glow from below/front — cold, blue-white, a little harsh. That's the '3am, still at it' look. Perfect for this shot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="40" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>If it's too dark</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Phone cameras get noisy in low light. If your face is barely visible, brighten the screen or move 10cm closer — don't add a lamp, it kills the mood.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="40" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Curtains</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Closed. No street light or daylight leaking in — it has to read as night.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>3 · OUTFIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="38" customHeight="1">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Vibe</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>'Been at this for hours.' Comfortable, lived-in, not styled. You just don't want it to look like you dressed up for a shoot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="38" customHeight="1">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Best pick</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>A plain dark hoodie or a plain tee — charcoal, black, deep grey. Solid colour, no big logos or bright prints.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="38" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>Pure white (glows/blows out against the dark), bright colours, busy patterns, anything that pulls the eye off your face.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="38" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Hoodie tip</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>If you own one, a hoodie is ideal here — hood down or half-up reads 'late night grind' instantly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="38" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Detail</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>Slightly messy hair is a plus, not a problem. This is the tired shot — a little dishevelled sells it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>4 · BODY LANGUAGE</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="36" customHeight="1">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Defeated, not dramatic. Heavy, slow, still. The camera should feel like it caught a real low moment, not a pose.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="36" customHeight="1">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Shoulders</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>Dropped and rounded forward. Let them sink — don't sit up straight.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="36" customHeight="1">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Head</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>Lowered. Either resting in one hand (palm on forehead / hand through hair) or hung down looking at the desk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="36" customHeight="1">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Hands</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>One hand up at your head OR both loose on the desk. Slow. No fidgeting, no phone, no typing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="36" customHeight="1">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Back</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>Slumped low in the chair, a little curled in. Small, not upright.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="36" customHeight="1">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Stillness</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>This is the whole shot. Hold nearly frozen for the full take — one slow breath, maybe one small head-shake or eyes-closed. That's it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="36" customHeight="1">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Do NOT</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>Look at the camera. Smile. Move fast. Perform 'tired' with big gestures. Under-act — stillness reads as exhausted; acting reads as fake.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>5 · THE 8 SECONDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="46" customHeight="1">
+      <c r="A41" s="30" t="inlineStr">
+        <is>
+          <t>Roll, then do almost nothing. Options, pick one: (a) sit slumped, head in hand, completely still, one slow breath; (b) rub your eyes / drag a hand down your face once, then go still; (c) stare at the screen, close your eyes for a beat, small shake of the head. Any of these, done SMALL and SLOW, is the shot. Record 3 takes and keep the stillest, most honest one. On-screen text lands here: "i almost deleted the whole thing."</t>
+        </is>
+      </c>
+    </row>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>BEFORE YOU ROLL — quick check</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="32" t="inlineStr">
+        <is>
+          <t>☐  Tripod locked, vertical, top third of frame dark</t>
+        </is>
+      </c>
+      <c r="B45" s="33" t="n"/>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="32" t="inlineStr">
+        <is>
+          <t>☐  Every light off except the laptop; bright screen up; brightness maxed, auto-brightness off</t>
+        </is>
+      </c>
+      <c r="B46" s="33" t="n"/>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="32" t="inlineStr">
+        <is>
+          <t>☐  Curtains closed</t>
+        </is>
+      </c>
+      <c r="B47" s="33" t="n"/>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="32" t="inlineStr">
+        <is>
+          <t>☐  Dark plain outfit on</t>
+        </is>
+      </c>
+      <c r="B48" s="33" t="n"/>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="32" t="inlineStr">
+        <is>
+          <t>☐  Do Not Disturb on; no notification lights</t>
+        </is>
+      </c>
+      <c r="B49" s="33" t="n"/>
+    </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="32" t="inlineStr">
+        <is>
+          <t>☐  Focus + exposure locked on your face</t>
+        </is>
+      </c>
+      <c r="B50" s="33" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A13:D13"/>
+  <mergeCells count="13">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A48:B48"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="A49:B49"/>
+    <mergeCell ref="A47:B47"/>
+    <mergeCell ref="A41:B43"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A50:B50"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rebalance the reel camera-forward now there's a tripod
Flips the build reel from 11 screen / 1 camera to 7 camera / 5 screen: the
grind and payoff are now carried by shots of the person, intercut with the
three screen moments that must stay screen — the error, the successful
build, and the app blending. Adds a Camera Setups sheet with five tripod
marks; the desk-shot lighting, wardrobe and body-language direction now
applies to every camera shot.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JLTsBRbD5LTCiR7DCK43kP
</commit_message>
<xml_diff>
--- a/memory-lane-reel.xlsx
+++ b/memory-lane-reel.xlsx
@@ -10,13 +10,14 @@
     <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Shot List" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Shot-by-Shot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Capture Guide" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="The Desk Shot" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Text &amp; Timing" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Edit Steps" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Music" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Take Tracker" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Post &amp; Caption" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Camera Setups" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Capture Guide" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="The Desk Shot" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Text &amp; Timing" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Edit Steps" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Music" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Take Tracker" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Post &amp; Caption" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -87,7 +88,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -132,6 +133,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FBE9EF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E4EBF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -194,7 +200,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -285,6 +291,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -671,6 +680,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -722,7 +732,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>1 (the desk shot). The other 11 are screen recordings.</t>
+          <t>7 camera shots on the tripod + 5 screen inserts (12 total).</t>
         </is>
       </c>
     </row>
@@ -774,6 +784,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
@@ -911,6 +922,260 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Take Tracker — tick as you shoot</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Fill the yellow cells. Aim for a keeper on every shot before you start editing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Shot</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>What</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Take 1</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Take 2</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Take 3</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Keeper?</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Open an empty file / blank VS Code project</t>
+        </is>
+      </c>
+      <c r="C5" s="28" t="inlineStr"/>
+      <c r="D5" s="28" t="inlineStr"/>
+      <c r="E5" s="28" t="inlineStr"/>
+      <c r="F5" s="28" t="inlineStr"/>
+      <c r="G5" s="29" t="inlineStr"/>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Your real code — scroll blend.ts / Orb.tsx</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="inlineStr"/>
+      <c r="D6" s="28" t="inlineStr"/>
+      <c r="E6" s="28" t="inlineStr"/>
+      <c r="F6" s="28" t="inlineStr"/>
+      <c r="G6" s="29" t="inlineStr"/>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>PowerShell — run the build command</t>
+        </is>
+      </c>
+      <c r="C7" s="28" t="inlineStr"/>
+      <c r="D7" s="28" t="inlineStr"/>
+      <c r="E7" s="28" t="inlineStr"/>
+      <c r="F7" s="28" t="inlineStr"/>
+      <c r="G7" s="29" t="inlineStr"/>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="27" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>EAS build logs streaming</t>
+        </is>
+      </c>
+      <c r="C8" s="28" t="inlineStr"/>
+      <c r="D8" s="28" t="inlineStr"/>
+      <c r="E8" s="28" t="inlineStr"/>
+      <c r="F8" s="28" t="inlineStr"/>
+      <c r="G8" s="29" t="inlineStr"/>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="27" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>The RED — a real / representative failure</t>
+        </is>
+      </c>
+      <c r="C9" s="28" t="inlineStr"/>
+      <c r="D9" s="28" t="inlineStr"/>
+      <c r="E9" s="28" t="inlineStr"/>
+      <c r="F9" s="28" t="inlineStr"/>
+      <c r="G9" s="29" t="inlineStr"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="27" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>A second, different error</t>
+        </is>
+      </c>
+      <c r="C10" s="28" t="inlineStr"/>
+      <c r="D10" s="28" t="inlineStr"/>
+      <c r="E10" s="28" t="inlineStr"/>
+      <c r="F10" s="28" t="inlineStr"/>
+      <c r="G10" s="29" t="inlineStr"/>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="27" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>git log — real late-night timestamps</t>
+        </is>
+      </c>
+      <c r="C11" s="28" t="inlineStr"/>
+      <c r="D11" s="28" t="inlineStr"/>
+      <c r="E11" s="28" t="inlineStr"/>
+      <c r="F11" s="28" t="inlineStr"/>
+      <c r="G11" s="29" t="inlineStr"/>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="27" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>YOU at the desk — the one human shot</t>
+        </is>
+      </c>
+      <c r="C12" s="28" t="inlineStr"/>
+      <c r="D12" s="28" t="inlineStr"/>
+      <c r="E12" s="28" t="inlineStr"/>
+      <c r="F12" s="28" t="inlineStr"/>
+      <c r="G12" s="29" t="inlineStr"/>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="27" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Build SUCCEEDED</t>
+        </is>
+      </c>
+      <c r="C13" s="28" t="inlineStr"/>
+      <c r="D13" s="28" t="inlineStr"/>
+      <c r="E13" s="28" t="inlineStr"/>
+      <c r="F13" s="28" t="inlineStr"/>
+      <c r="G13" s="29" t="inlineStr"/>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="27" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Install on a real phone</t>
+        </is>
+      </c>
+      <c r="C14" s="28" t="inlineStr"/>
+      <c r="D14" s="28" t="inlineStr"/>
+      <c r="E14" s="28" t="inlineStr"/>
+      <c r="F14" s="28" t="inlineStr"/>
+      <c r="G14" s="29" t="inlineStr"/>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="27" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>The app works — fill an orb</t>
+        </is>
+      </c>
+      <c r="C15" s="28" t="inlineStr"/>
+      <c r="D15" s="28" t="inlineStr"/>
+      <c r="E15" s="28" t="inlineStr"/>
+      <c r="F15" s="28" t="inlineStr"/>
+      <c r="G15" s="29" t="inlineStr"/>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="27" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Your handle + link over an orb</t>
+        </is>
+      </c>
+      <c r="C16" s="28" t="inlineStr"/>
+      <c r="D16" s="28" t="inlineStr"/>
+      <c r="E16" s="28" t="inlineStr"/>
+      <c r="F16" s="28" t="inlineStr"/>
+      <c r="G16" s="29" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1064,33 +1329,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
     <col width="6" customWidth="1" min="4" max="4"/>
     <col width="6" customWidth="1" min="5" max="5"/>
     <col width="6" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="6" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Shot List — master</t>
+          <t>Shot List — camera-forward</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Blue Duration cells are yours to change — every timecode re-syncs. All others read at a glance.</t>
+          <t>7 camera shots on the tripod, 5 screen inserts. The 3 screen shots that must stay screen: 5 (error), 9 (built), 11 (app works). Blue Dur cells re-sync.</t>
         </is>
       </c>
     </row>
@@ -1107,51 +1373,56 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>Cam/Screen</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
+          <t>Mark</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
           <t>Dur</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Start</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>End</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Timecode</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>What you capture</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>On-screen text</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>Text pos</t>
-        </is>
-      </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
+          <t>Pos</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
           <t>Transition</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="42" customHeight="1">
+    <row r="5" ht="44" customHeight="1">
       <c r="A5" s="7" t="n">
         <v>1</v>
       </c>
@@ -1160,47 +1431,52 @@
           <t>GRIND</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
-        <is>
-          <t>screen rec</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="n">
+      <c r="C5" s="34" t="inlineStr">
+        <is>
+          <t>CAMERA</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="E5" s="7" t="n">
+      <c r="F5" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="7">
-        <f>E5+D5</f>
+      <c r="G5" s="7">
+        <f>F5+E5</f>
         <v/>
       </c>
-      <c r="G5" s="7">
-        <f>"0:"&amp;TEXT(E5,"00")&amp;"-0:"&amp;TEXT(F5,"00")</f>
+      <c r="H5" s="7">
+        <f>"0:"&amp;TEXT(F5,"00")&amp;"-0:"&amp;TEXT(G5,"00")</f>
         <v/>
       </c>
-      <c r="H5" s="9" t="inlineStr">
-        <is>
-          <t>Open an empty file / blank VS Code project</t>
-        </is>
-      </c>
       <c r="I5" s="9" t="inlineStr">
         <is>
+          <t>Wide, behind you — you sit down at the dark desk, laptop glowing</t>
+        </is>
+      </c>
+      <c r="J5" s="9" t="inlineStr">
+        <is>
           <t>3 days ago this was nothing</t>
         </is>
       </c>
-      <c r="J5" s="7" t="inlineStr">
-        <is>
-          <t>top-centre</t>
-        </is>
-      </c>
-      <c r="K5" s="9" t="inlineStr">
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>top</t>
+        </is>
+      </c>
+      <c r="L5" s="9" t="inlineStr">
         <is>
           <t>hard cut</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="42" customHeight="1">
+    <row r="6" ht="44" customHeight="1">
       <c r="A6" s="7" t="n">
         <v>2</v>
       </c>
@@ -1209,48 +1485,53 @@
           <t>GRIND</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
-        <is>
-          <t>screen rec</t>
-        </is>
-      </c>
-      <c r="D6" s="10" t="n">
+      <c r="C6" s="34" t="inlineStr">
+        <is>
+          <t>CAMERA</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="E6" s="7">
-        <f>F5</f>
+      <c r="F6" s="7">
+        <f>G5</f>
         <v/>
       </c>
-      <c r="F6" s="7">
-        <f>E6+D6</f>
+      <c r="G6" s="7">
+        <f>F6+E6</f>
         <v/>
       </c>
-      <c r="G6" s="7">
-        <f>"0:"&amp;TEXT(E6,"00")&amp;"-0:"&amp;TEXT(F6,"00")</f>
+      <c r="H6" s="7">
+        <f>"0:"&amp;TEXT(F6,"00")&amp;"-0:"&amp;TEXT(G6,"00")</f>
         <v/>
       </c>
-      <c r="H6" s="9" t="inlineStr">
-        <is>
-          <t>Your real code — scroll blend.ts / Orb.tsx</t>
-        </is>
-      </c>
       <c r="I6" s="9" t="inlineStr">
         <is>
+          <t>Over-shoulder — your hands typing, code on the screen</t>
+        </is>
+      </c>
+      <c r="J6" s="9" t="inlineStr">
+        <is>
           <t>so i started building</t>
         </is>
       </c>
-      <c r="J6" s="7" t="inlineStr">
-        <is>
-          <t>top-centre</t>
-        </is>
-      </c>
-      <c r="K6" s="9" t="inlineStr">
+      <c r="K6" s="7" t="inlineStr">
+        <is>
+          <t>top</t>
+        </is>
+      </c>
+      <c r="L6" s="9" t="inlineStr">
         <is>
           <t>hard cut</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="42" customHeight="1">
+    <row r="7" ht="44" customHeight="1">
       <c r="A7" s="7" t="n">
         <v>3</v>
       </c>
@@ -1259,48 +1540,53 @@
           <t>GRIND</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>screen rec</t>
-        </is>
-      </c>
-      <c r="D7" s="10" t="n">
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>SCREEN</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="E7" s="7">
-        <f>F6</f>
+      <c r="F7" s="7">
+        <f>G6</f>
         <v/>
       </c>
-      <c r="F7" s="7">
-        <f>E7+D7</f>
+      <c r="G7" s="7">
+        <f>F7+E7</f>
         <v/>
       </c>
-      <c r="G7" s="7">
-        <f>"0:"&amp;TEXT(E7,"00")&amp;"-0:"&amp;TEXT(F7,"00")</f>
+      <c r="H7" s="7">
+        <f>"0:"&amp;TEXT(F7,"00")&amp;"-0:"&amp;TEXT(G7,"00")</f>
         <v/>
       </c>
-      <c r="H7" s="9" t="inlineStr">
-        <is>
-          <t>PowerShell — run the build command</t>
-        </is>
-      </c>
       <c r="I7" s="9" t="inlineStr">
         <is>
+          <t>Screen insert — the build command</t>
+        </is>
+      </c>
+      <c r="J7" s="9" t="inlineStr">
+        <is>
           <t>one command to ship it</t>
         </is>
       </c>
-      <c r="J7" s="7" t="inlineStr">
-        <is>
-          <t>lower-centre</t>
-        </is>
-      </c>
-      <c r="K7" s="9" t="inlineStr">
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="L7" s="9" t="inlineStr">
         <is>
           <t>hard cut</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="42" customHeight="1">
+    <row r="8" ht="44" customHeight="1">
       <c r="A8" s="7" t="n">
         <v>4</v>
       </c>
@@ -1309,48 +1595,53 @@
           <t>GRIND</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>screen rec</t>
-        </is>
-      </c>
-      <c r="D8" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="E8" s="7">
-        <f>F7</f>
+      <c r="C8" s="34" t="inlineStr">
+        <is>
+          <t>CAMERA</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" s="7">
+        <f>G7</f>
         <v/>
       </c>
-      <c r="F8" s="7">
-        <f>E8+D8</f>
+      <c r="G8" s="7">
+        <f>F8+E8</f>
         <v/>
       </c>
-      <c r="G8" s="7">
-        <f>"0:"&amp;TEXT(E8,"00")&amp;"-0:"&amp;TEXT(F8,"00")</f>
+      <c r="H8" s="7">
+        <f>"0:"&amp;TEXT(F8,"00")&amp;"-0:"&amp;TEXT(G8,"00")</f>
         <v/>
       </c>
-      <c r="H8" s="9" t="inlineStr">
-        <is>
-          <t>EAS build logs streaming</t>
-        </is>
-      </c>
       <c r="I8" s="9" t="inlineStr">
         <is>
+          <t>Your face, lit by the screen — watching, waiting</t>
+        </is>
+      </c>
+      <c r="J8" s="9" t="inlineStr">
+        <is>
           <t>or so i thought</t>
         </is>
       </c>
-      <c r="J8" s="7" t="inlineStr">
-        <is>
-          <t>top-centre</t>
-        </is>
-      </c>
-      <c r="K8" s="9" t="inlineStr">
+      <c r="K8" s="7" t="inlineStr">
+        <is>
+          <t>top</t>
+        </is>
+      </c>
+      <c r="L8" s="9" t="inlineStr">
         <is>
           <t>hard cut</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="42" customHeight="1">
+    <row r="9" ht="44" customHeight="1">
       <c r="A9" s="7" t="n">
         <v>5</v>
       </c>
@@ -1359,48 +1650,53 @@
           <t>GRIND</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>screen rec</t>
-        </is>
-      </c>
-      <c r="D9" s="10" t="n">
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>SCREEN</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="E9" s="7">
-        <f>F8</f>
+      <c r="F9" s="7">
+        <f>G8</f>
         <v/>
       </c>
-      <c r="F9" s="7">
-        <f>E9+D9</f>
+      <c r="G9" s="7">
+        <f>F9+E9</f>
         <v/>
       </c>
-      <c r="G9" s="7">
-        <f>"0:"&amp;TEXT(E9,"00")&amp;"-0:"&amp;TEXT(F9,"00")</f>
+      <c r="H9" s="7">
+        <f>"0:"&amp;TEXT(F9,"00")&amp;"-0:"&amp;TEXT(G9,"00")</f>
         <v/>
       </c>
-      <c r="H9" s="9" t="inlineStr">
-        <is>
-          <t>The RED — a real / representative failure</t>
-        </is>
-      </c>
       <c r="I9" s="9" t="inlineStr">
         <is>
+          <t>Screen insert — the RED error</t>
+        </is>
+      </c>
+      <c r="J9" s="9" t="inlineStr">
+        <is>
           <t>it broke.</t>
         </is>
       </c>
-      <c r="J9" s="7" t="inlineStr">
+      <c r="K9" s="7" t="inlineStr">
         <is>
           <t>centre</t>
         </is>
       </c>
-      <c r="K9" s="9" t="inlineStr">
-        <is>
-          <t>quick flash / shake</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="42" customHeight="1">
+      <c r="L9" s="9" t="inlineStr">
+        <is>
+          <t>quick flash</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="44" customHeight="1">
       <c r="A10" s="7" t="n">
         <v>6</v>
       </c>
@@ -1409,48 +1705,53 @@
           <t>GRIND</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>screen rec</t>
-        </is>
-      </c>
-      <c r="D10" s="10" t="n">
+      <c r="C10" s="34" t="inlineStr">
+        <is>
+          <t>CAMERA</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="E10" s="7">
-        <f>F9</f>
+      <c r="F10" s="7">
+        <f>G9</f>
         <v/>
       </c>
-      <c r="F10" s="7">
-        <f>E10+D10</f>
+      <c r="G10" s="7">
+        <f>F10+E10</f>
         <v/>
       </c>
-      <c r="G10" s="7">
-        <f>"0:"&amp;TEXT(E10,"00")&amp;"-0:"&amp;TEXT(F10,"00")</f>
+      <c r="H10" s="7">
+        <f>"0:"&amp;TEXT(F10,"00")&amp;"-0:"&amp;TEXT(G10,"00")</f>
         <v/>
       </c>
-      <c r="H10" s="9" t="inlineStr">
-        <is>
-          <t>A second, different error</t>
-        </is>
-      </c>
       <c r="I10" s="9" t="inlineStr">
         <is>
-          <t>and broke again.</t>
-        </is>
-      </c>
-      <c r="J10" s="7" t="inlineStr">
-        <is>
-          <t>centre</t>
-        </is>
-      </c>
-      <c r="K10" s="9" t="inlineStr">
+          <t>Mid, side-on — you react to the error</t>
+        </is>
+      </c>
+      <c r="J10" s="9" t="inlineStr">
+        <is>
+          <t>and again.</t>
+        </is>
+      </c>
+      <c r="K10" s="7" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="L10" s="9" t="inlineStr">
         <is>
           <t>quick flash</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="42" customHeight="1">
+    <row r="11" ht="44" customHeight="1">
       <c r="A11" s="7" t="n">
         <v>7</v>
       </c>
@@ -1459,48 +1760,53 @@
           <t>GRIND</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>screen rec</t>
-        </is>
-      </c>
-      <c r="D11" s="10" t="n">
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>SCREEN</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="E11" s="7">
-        <f>F10</f>
+      <c r="F11" s="7">
+        <f>G10</f>
         <v/>
       </c>
-      <c r="F11" s="7">
-        <f>E11+D11</f>
+      <c r="G11" s="7">
+        <f>F11+E11</f>
         <v/>
       </c>
-      <c r="G11" s="7">
-        <f>"0:"&amp;TEXT(E11,"00")&amp;"-0:"&amp;TEXT(F11,"00")</f>
+      <c r="H11" s="7">
+        <f>"0:"&amp;TEXT(F11,"00")&amp;"-0:"&amp;TEXT(G11,"00")</f>
         <v/>
       </c>
-      <c r="H11" s="9" t="inlineStr">
-        <is>
-          <t>git log — real late-night timestamps</t>
-        </is>
-      </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
+          <t>Screen insert — git log, late timestamps</t>
+        </is>
+      </c>
+      <c r="J11" s="9" t="inlineStr">
+        <is>
           <t>more nights than i'd admit</t>
         </is>
       </c>
-      <c r="J11" s="7" t="inlineStr">
+      <c r="K11" s="7" t="inlineStr">
         <is>
           <t>top-left</t>
         </is>
       </c>
-      <c r="K11" s="9" t="inlineStr">
+      <c r="L11" s="9" t="inlineStr">
         <is>
           <t>hard cut</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="42" customHeight="1">
+    <row r="12" ht="44" customHeight="1">
       <c r="A12" s="7" t="n">
         <v>8</v>
       </c>
@@ -1509,48 +1815,53 @@
           <t>HUMAN</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>camera</t>
-        </is>
-      </c>
-      <c r="D12" s="10" t="n">
+      <c r="C12" s="34" t="inlineStr">
+        <is>
+          <t>CAMERA</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="E12" s="7">
-        <f>F11</f>
+      <c r="F12" s="7">
+        <f>G11</f>
         <v/>
       </c>
-      <c r="F12" s="7">
-        <f>E12+D12</f>
+      <c r="G12" s="7">
+        <f>F12+E12</f>
         <v/>
       </c>
-      <c r="G12" s="7">
-        <f>"0:"&amp;TEXT(E12,"00")&amp;"-0:"&amp;TEXT(F12,"00")</f>
+      <c r="H12" s="7">
+        <f>"0:"&amp;TEXT(F12,"00")&amp;"-0:"&amp;TEXT(G12,"00")</f>
         <v/>
       </c>
-      <c r="H12" s="9" t="inlineStr">
-        <is>
-          <t>YOU at the desk — the one human shot</t>
-        </is>
-      </c>
       <c r="I12" s="9" t="inlineStr">
         <is>
-          <t>i almost deleted the whole thing</t>
-        </is>
-      </c>
-      <c r="J12" s="7" t="inlineStr">
-        <is>
-          <t>lower-centre</t>
-        </is>
-      </c>
-      <c r="K12" s="9" t="inlineStr">
-        <is>
-          <t>slow cut (breath)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="42" customHeight="1">
+          <t>THE desk shot — slumped, tired, still</t>
+        </is>
+      </c>
+      <c r="J12" s="9" t="inlineStr">
+        <is>
+          <t>i almost gave up on it</t>
+        </is>
+      </c>
+      <c r="K12" s="7" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="L12" s="9" t="inlineStr">
+        <is>
+          <t>slow cut</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="44" customHeight="1">
       <c r="A13" s="11" t="n">
         <v>9</v>
       </c>
@@ -1559,48 +1870,53 @@
           <t>TURN</t>
         </is>
       </c>
-      <c r="C13" s="13" t="inlineStr">
-        <is>
-          <t>screen rec</t>
-        </is>
-      </c>
-      <c r="D13" s="10" t="n">
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>SCREEN</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="11">
-        <f>F12</f>
+      <c r="F13" s="11">
+        <f>G12</f>
         <v/>
       </c>
-      <c r="F13" s="11">
-        <f>E13+D13</f>
+      <c r="G13" s="11">
+        <f>F13+E13</f>
         <v/>
       </c>
-      <c r="G13" s="11">
-        <f>"0:"&amp;TEXT(E13,"00")&amp;"-0:"&amp;TEXT(F13,"00")</f>
+      <c r="H13" s="11">
+        <f>"0:"&amp;TEXT(F13,"00")&amp;"-0:"&amp;TEXT(G13,"00")</f>
         <v/>
       </c>
-      <c r="H13" s="13" t="inlineStr">
-        <is>
-          <t>Build SUCCEEDED</t>
-        </is>
-      </c>
       <c r="I13" s="13" t="inlineStr">
         <is>
+          <t>Screen insert — build SUCCEEDED</t>
+        </is>
+      </c>
+      <c r="J13" s="13" t="inlineStr">
+        <is>
           <t>then — it built.</t>
         </is>
       </c>
-      <c r="J13" s="11" t="inlineStr">
+      <c r="K13" s="11" t="inlineStr">
         <is>
           <t>centre</t>
         </is>
       </c>
-      <c r="K13" s="13" t="inlineStr">
-        <is>
-          <t>cut on the beat</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="42" customHeight="1">
+      <c r="L13" s="13" t="inlineStr">
+        <is>
+          <t>cut on beat</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="44" customHeight="1">
       <c r="A14" s="11" t="n">
         <v>10</v>
       </c>
@@ -1609,48 +1925,53 @@
           <t>TURN</t>
         </is>
       </c>
-      <c r="C14" s="13" t="inlineStr">
-        <is>
-          <t>screen rec / phone</t>
-        </is>
-      </c>
-      <c r="D14" s="10" t="n">
+      <c r="C14" s="34" t="inlineStr">
+        <is>
+          <t>CAMERA</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="E14" s="11">
-        <f>F13</f>
+      <c r="F14" s="11">
+        <f>G13</f>
         <v/>
       </c>
-      <c r="F14" s="11">
-        <f>E14+D14</f>
+      <c r="G14" s="11">
+        <f>F14+E14</f>
         <v/>
       </c>
-      <c r="G14" s="11">
-        <f>"0:"&amp;TEXT(E14,"00")&amp;"-0:"&amp;TEXT(F14,"00")</f>
+      <c r="H14" s="11">
+        <f>"0:"&amp;TEXT(F14,"00")&amp;"-0:"&amp;TEXT(G14,"00")</f>
         <v/>
       </c>
-      <c r="H14" s="13" t="inlineStr">
-        <is>
-          <t>Install on a real phone</t>
-        </is>
-      </c>
       <c r="I14" s="13" t="inlineStr">
         <is>
+          <t>You + your phone — it installs</t>
+        </is>
+      </c>
+      <c r="J14" s="13" t="inlineStr">
+        <is>
           <t>it installed on a real phone</t>
         </is>
       </c>
-      <c r="J14" s="11" t="inlineStr">
-        <is>
-          <t>top-centre</t>
-        </is>
-      </c>
-      <c r="K14" s="13" t="inlineStr">
+      <c r="K14" s="11" t="inlineStr">
+        <is>
+          <t>top</t>
+        </is>
+      </c>
+      <c r="L14" s="13" t="inlineStr">
         <is>
           <t>hard cut</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="42" customHeight="1">
+    <row r="15" ht="44" customHeight="1">
       <c r="A15" s="14" t="n">
         <v>11</v>
       </c>
@@ -1659,48 +1980,53 @@
           <t>GIFT</t>
         </is>
       </c>
-      <c r="C15" s="16" t="inlineStr">
-        <is>
-          <t>screen rec</t>
-        </is>
-      </c>
-      <c r="D15" s="10" t="n">
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>SCREEN</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="E15" s="14">
-        <f>F14</f>
+      <c r="F15" s="14">
+        <f>G14</f>
         <v/>
       </c>
-      <c r="F15" s="14">
-        <f>E15+D15</f>
+      <c r="G15" s="14">
+        <f>F15+E15</f>
         <v/>
       </c>
-      <c r="G15" s="14">
-        <f>"0:"&amp;TEXT(E15,"00")&amp;"-0:"&amp;TEXT(F15,"00")</f>
+      <c r="H15" s="14">
+        <f>"0:"&amp;TEXT(F15,"00")&amp;"-0:"&amp;TEXT(G15,"00")</f>
         <v/>
       </c>
-      <c r="H15" s="16" t="inlineStr">
-        <is>
-          <t>The app works — fill an orb</t>
-        </is>
-      </c>
       <c r="I15" s="16" t="inlineStr">
         <is>
+          <t>Screen insert — the app WORKS</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
           <t>and it actually works</t>
         </is>
       </c>
-      <c r="J15" s="14" t="inlineStr">
-        <is>
-          <t>top-centre</t>
-        </is>
-      </c>
-      <c r="K15" s="16" t="inlineStr">
+      <c r="K15" s="14" t="inlineStr">
+        <is>
+          <t>top</t>
+        </is>
+      </c>
+      <c r="L15" s="16" t="inlineStr">
         <is>
           <t>slow</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="42" customHeight="1">
+    <row r="16" ht="44" customHeight="1">
       <c r="A16" s="14" t="n">
         <v>12</v>
       </c>
@@ -1709,42 +2035,47 @@
           <t>GIFT</t>
         </is>
       </c>
-      <c r="C16" s="16" t="inlineStr">
-        <is>
-          <t>designed card</t>
-        </is>
-      </c>
-      <c r="D16" s="10" t="n">
+      <c r="C16" s="34" t="inlineStr">
+        <is>
+          <t>CAMERA</t>
+        </is>
+      </c>
+      <c r="D16" s="14" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="E16" s="14">
-        <f>F15</f>
+      <c r="F16" s="14">
+        <f>G15</f>
         <v/>
       </c>
-      <c r="F16" s="14">
-        <f>E16+D16</f>
+      <c r="G16" s="14">
+        <f>F16+E16</f>
         <v/>
       </c>
-      <c r="G16" s="14">
-        <f>"0:"&amp;TEXT(E16,"00")&amp;"-0:"&amp;TEXT(F16,"00")</f>
+      <c r="H16" s="14">
+        <f>"0:"&amp;TEXT(F16,"00")&amp;"-0:"&amp;TEXT(G16,"00")</f>
         <v/>
       </c>
-      <c r="H16" s="16" t="inlineStr">
-        <is>
-          <t>Your handle + link over an orb</t>
-        </is>
-      </c>
       <c r="I16" s="16" t="inlineStr">
         <is>
+          <t>You + phone, looking at it — the end</t>
+        </is>
+      </c>
+      <c r="J16" s="16" t="inlineStr">
+        <is>
           <t>i built this. it's live 👇</t>
         </is>
       </c>
-      <c r="J16" s="14" t="inlineStr">
+      <c r="K16" s="14" t="inlineStr">
         <is>
           <t>centre</t>
         </is>
       </c>
-      <c r="K16" s="16" t="inlineStr">
+      <c r="L16" s="16" t="inlineStr">
         <is>
           <t>hold to end</t>
         </is>
@@ -1753,25 +2084,26 @@
     <row r="17">
       <c r="A17" s="17" t="n"/>
       <c r="B17" s="17" t="n"/>
-      <c r="C17" s="18" t="inlineStr">
+      <c r="C17" s="17" t="n"/>
+      <c r="D17" s="18" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="D17" s="18">
-        <f>SUM(D5:D16)</f>
+      <c r="E17" s="18">
+        <f>SUM(E5:E16)</f>
         <v/>
       </c>
-      <c r="E17" s="17" t="n"/>
       <c r="F17" s="17" t="n"/>
-      <c r="G17" s="18">
-        <f>"0:"&amp;TEXT(SUM(D5:D16),"00")</f>
+      <c r="G17" s="17" t="n"/>
+      <c r="H17" s="18">
+        <f>"0:"&amp;TEXT(SUM(E5:E16),"00")</f>
         <v/>
       </c>
-      <c r="H17" s="17" t="n"/>
       <c r="I17" s="17" t="n"/>
       <c r="J17" s="17" t="n"/>
       <c r="K17" s="17" t="n"/>
+      <c r="L17" s="17" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1784,7 +2116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B63"/>
+  <dimension ref="A1:B74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1794,25 +2126,25 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Shot-by-Shot — follow while recording</t>
+          <t>Shot-by-Shot</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>One block per shot. Everything you need is here — no jumping between sheets.</t>
+          <t>Follow while shooting. CAMERA shots use the tripod marks (see Camera Setups). SCREEN shots are recorded at the laptop.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="19" t="inlineStr">
         <is>
-          <t>SHOT 1  ·  GRIND  ·  3s  ·  SCREEN REC</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="26" customHeight="1">
+          <t>SHOT 1  ·  GRIND  ·  3s  ·  CAMERA  ·  MARK A</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
       <c r="A5" s="20" t="inlineStr">
         <is>
           <t>Capture</t>
@@ -1820,7 +2152,7 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Open an empty file / blank VS Code project</t>
+          <t>Wide, behind you — you sit down at the dark desk, laptop glowing</t>
         </is>
       </c>
     </row>
@@ -1832,11 +2164,11 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Start on a truly empty editor — one blank file, file tree hidden. Sit on it 1s, then the first line of code appears (paste/type one import).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="26" customHeight="1">
+          <t>You come into frame and sit, hands to the keyboard. Room dark, screen lit. Establishes 'a person, alone, starting.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
       <c r="A7" s="20" t="inlineStr">
         <is>
           <t>On-screen text</t>
@@ -1844,14 +2176,14 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>"3 days ago this was nothing"  —  top-centre</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="26" customHeight="1">
+          <t>"3 days ago this was nothing"  —  top</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
       <c r="A8" s="20" t="inlineStr">
         <is>
-          <t>Transition out</t>
+          <t>Cut out</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
@@ -1860,276 +2192,221 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>SHOT 2  ·  GRIND  ·  2s  ·  SCREEN REC</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="26" customHeight="1">
-      <c r="A10" s="20" t="inlineStr">
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>SHOT 2  ·  GRIND  ·  2s  ·  CAMERA  ·  MARK B</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>Capture</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>Your real code — scroll blend.ts / Orb.tsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="44" customHeight="1">
-      <c r="A11" s="20" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Over-shoulder — your hands typing, code on the screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="44" customHeight="1">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>Do this</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>Slow, even scroll through YOUR file (from reel-props). Dark theme, font ~18-20pt. Don't race it — let it read as real work.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="26" customHeight="1">
-      <c r="A12" s="20" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Shoot past your shoulder so BOTH your hands on the keys and the code on screen are in frame. Real typing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>On-screen text</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>"so i started building"  —  top-centre</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="26" customHeight="1">
-      <c r="A13" s="20" t="inlineStr">
-        <is>
-          <t>Transition out</t>
-        </is>
-      </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
+          <t>"so i started building"  —  top</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="20" t="inlineStr">
+        <is>
+          <t>Cut out</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
           <t>hard cut</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="19" t="inlineStr">
-        <is>
-          <t>SHOT 3  ·  GRIND  ·  2s  ·  SCREEN REC</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="26" customHeight="1">
-      <c r="A15" s="20" t="inlineStr">
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="19" t="inlineStr">
+        <is>
+          <t>SHOT 3  ·  GRIND  ·  2s  ·  SCREEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="20" t="inlineStr">
         <is>
           <t>Capture</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>PowerShell — run the build command</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="44" customHeight="1">
-      <c r="A16" s="20" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Screen insert — the build command</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="44" customHeight="1">
+      <c r="A18" s="20" t="inlineStr">
         <is>
           <t>Do this</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>Terminal full-screen. Type and run:  eas build --platform android --profile preview  — capture the keystrokes and the Enter.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="26" customHeight="1">
-      <c r="A17" s="20" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Terminal: run  eas build --platform android --profile preview. A clean screen recording, no camera.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="20" t="inlineStr">
         <is>
           <t>On-screen text</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>"one command to ship it"  —  lower-centre</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="26" customHeight="1">
-      <c r="A18" s="20" t="inlineStr">
-        <is>
-          <t>Transition out</t>
-        </is>
-      </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>"one command to ship it"  —  lower</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="20" t="inlineStr">
+        <is>
+          <t>Cut out</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>hard cut</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="19" t="inlineStr">
-        <is>
-          <t>SHOT 4  ·  GRIND  ·  3s  ·  SCREEN REC</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="26" customHeight="1">
-      <c r="A20" s="20" t="inlineStr">
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="19" t="inlineStr">
+        <is>
+          <t>SHOT 4  ·  GRIND  ·  2s  ·  CAMERA  ·  MARK C</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="20" t="inlineStr">
         <is>
           <t>Capture</t>
         </is>
       </c>
-      <c r="B20" s="9" t="inlineStr">
-        <is>
-          <t>EAS build logs streaming</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="44" customHeight="1">
-      <c r="A21" s="20" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Your face, lit by the screen — watching, waiting</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="44" customHeight="1">
+      <c r="A24" s="20" t="inlineStr">
         <is>
           <t>Do this</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>The build output scrolling — Gradle tasks, linking, compiling. Use 03-build-log.txt in a terminal, OR your real EAS page. Let it stream.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="26" customHeight="1">
-      <c r="A22" s="20" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Tight-ish on your face, side-lit by the laptop. You're watching the build, focused, a little tense. No words.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="20" t="inlineStr">
         <is>
           <t>On-screen text</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>"or so i thought"  —  top-centre</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="26" customHeight="1">
-      <c r="A23" s="20" t="inlineStr">
-        <is>
-          <t>Transition out</t>
-        </is>
-      </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>"or so i thought"  —  top</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="24" customHeight="1">
+      <c r="A26" s="20" t="inlineStr">
+        <is>
+          <t>Cut out</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
         <is>
           <t>hard cut</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="19" t="inlineStr">
-        <is>
-          <t>SHOT 5  ·  GRIND  ·  3s  ·  SCREEN REC</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="26" customHeight="1">
-      <c r="A25" s="20" t="inlineStr">
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="19" t="inlineStr">
+        <is>
+          <t>SHOT 5  ·  GRIND  ·  3s  ·  SCREEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="24" customHeight="1">
+      <c r="A29" s="20" t="inlineStr">
         <is>
           <t>Capture</t>
         </is>
       </c>
-      <c r="B25" s="9" t="inlineStr">
-        <is>
-          <t>The RED — a real / representative failure</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="44" customHeight="1">
-      <c r="A26" s="20" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>Screen insert — the RED error</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="44" customHeight="1">
+      <c r="A30" s="20" t="inlineStr">
         <is>
           <t>Do this</t>
         </is>
       </c>
-      <c r="B26" s="9" t="inlineStr">
-        <is>
-          <t>04-error.txt, or your real gradle error. Frame so the red FAILED / error text fills the shot. HOLD 3s — this is the low beat starting.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="26" customHeight="1">
-      <c r="A27" s="20" t="inlineStr">
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>04-error.txt or your real gradle failure. Frame tight on the red FAILED. Hold. This is the low beat starting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="24" customHeight="1">
+      <c r="A31" s="20" t="inlineStr">
         <is>
           <t>On-screen text</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B31" s="9" t="inlineStr">
         <is>
           <t>"it broke."  —  centre</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="26" customHeight="1">
-      <c r="A28" s="20" t="inlineStr">
-        <is>
-          <t>Transition out</t>
-        </is>
-      </c>
-      <c r="B28" s="9" t="inlineStr">
-        <is>
-          <t>quick flash / shake</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="19" t="inlineStr">
-        <is>
-          <t>SHOT 6  ·  GRIND  ·  2s  ·  SCREEN REC</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="26" customHeight="1">
-      <c r="A30" s="20" t="inlineStr">
-        <is>
-          <t>Capture</t>
-        </is>
-      </c>
-      <c r="B30" s="9" t="inlineStr">
-        <is>
-          <t>A second, different error</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="44" customHeight="1">
-      <c r="A31" s="20" t="inlineStr">
-        <is>
-          <t>Do this</t>
-        </is>
-      </c>
-      <c r="B31" s="9" t="inlineStr">
-        <is>
-          <t>05-error-2.txt — a different error type (metro / dependency). Different red, so it reads as 'again', not the same shot repeated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="26" customHeight="1">
+    <row r="32" ht="24" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>On-screen text</t>
+          <t>Cut out</t>
         </is>
       </c>
       <c r="B32" s="9" t="inlineStr">
-        <is>
-          <t>"and broke again."  —  centre</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="26" customHeight="1">
-      <c r="A33" s="20" t="inlineStr">
-        <is>
-          <t>Transition out</t>
-        </is>
-      </c>
-      <c r="B33" s="9" t="inlineStr">
         <is>
           <t>quick flash</t>
         </is>
@@ -2138,11 +2415,11 @@
     <row r="34" ht="22" customHeight="1">
       <c r="A34" s="19" t="inlineStr">
         <is>
-          <t>SHOT 7  ·  GRIND  ·  2s  ·  SCREEN REC</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="26" customHeight="1">
+          <t>SHOT 6  ·  GRIND  ·  2s  ·  CAMERA  ·  MARK D</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="24" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
           <t>Capture</t>
@@ -2150,7 +2427,7 @@
       </c>
       <c r="B35" s="9" t="inlineStr">
         <is>
-          <t>git log — real late-night timestamps</t>
+          <t>Mid, side-on — you react to the error</t>
         </is>
       </c>
     </row>
@@ -2162,11 +2439,11 @@
       </c>
       <c r="B36" s="9" t="inlineStr">
         <is>
-          <t>Run:  git log --pretty=format:'%h %ad %s' --date=format:'%H:%M'  — scroll your real commit times. SEE TEXT SHEET re: the on-screen claim.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="26" customHeight="1">
+          <t>You lean back and drag a hand down your face, or hands on head. One real, frustrated movement. Don't overplay it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="24" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
           <t>On-screen text</t>
@@ -2174,292 +2451,347 @@
       </c>
       <c r="B37" s="9" t="inlineStr">
         <is>
+          <t>"and again."  —  lower</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="24" customHeight="1">
+      <c r="A38" s="20" t="inlineStr">
+        <is>
+          <t>Cut out</t>
+        </is>
+      </c>
+      <c r="B38" s="9" t="inlineStr">
+        <is>
+          <t>quick flash</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="19" t="inlineStr">
+        <is>
+          <t>SHOT 7  ·  GRIND  ·  2s  ·  SCREEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="24" customHeight="1">
+      <c r="A41" s="20" t="inlineStr">
+        <is>
+          <t>Capture</t>
+        </is>
+      </c>
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>Screen insert — git log, late timestamps</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="44" customHeight="1">
+      <c r="A42" s="20" t="inlineStr">
+        <is>
+          <t>Do this</t>
+        </is>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>git log --pretty=format:'%h %ad %s' --date=format:'%H:%M'  — scroll your real commit times.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="24" customHeight="1">
+      <c r="A43" s="20" t="inlineStr">
+        <is>
+          <t>On-screen text</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="inlineStr">
+        <is>
           <t>"more nights than i'd admit"  —  top-left</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="26" customHeight="1">
-      <c r="A38" s="20" t="inlineStr">
-        <is>
-          <t>Transition out</t>
-        </is>
-      </c>
-      <c r="B38" s="9" t="inlineStr">
+    <row r="44" ht="24" customHeight="1">
+      <c r="A44" s="20" t="inlineStr">
+        <is>
+          <t>Cut out</t>
+        </is>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
         <is>
           <t>hard cut</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="22" customHeight="1">
-      <c r="A39" s="19" t="inlineStr">
-        <is>
-          <t>SHOT 8  ·  HUMAN  ·  3s  ·  CAMERA</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="26" customHeight="1">
-      <c r="A40" s="20" t="inlineStr">
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="19" t="inlineStr">
+        <is>
+          <t>SHOT 8  ·  HUMAN  ·  3s  ·  CAMERA  ·  MARK A</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="24" customHeight="1">
+      <c r="A47" s="20" t="inlineStr">
         <is>
           <t>Capture</t>
         </is>
       </c>
-      <c r="B40" s="9" t="inlineStr">
-        <is>
-          <t>YOU at the desk — the one human shot</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="44" customHeight="1">
-      <c r="A41" s="20" t="inlineStr">
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>THE desk shot — slumped, tired, still</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="44" customHeight="1">
+      <c r="A48" s="20" t="inlineStr">
         <is>
           <t>Do this</t>
         </is>
       </c>
-      <c r="B41" s="9" t="inlineStr">
-        <is>
-          <t>Tripod behind you, low, dark room, only the laptop lighting your face. Sit slumped, head in hand, still. One 8s take, use the calmest.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="26" customHeight="1">
-      <c r="A42" s="20" t="inlineStr">
+      <c r="B48" s="9" t="inlineStr">
+        <is>
+          <t>Back to the wide/behind mark. Slumped low, head in one hand, completely still. The emotional bottom. See 'The Desk Shot' sheet for full direction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="24" customHeight="1">
+      <c r="A49" s="20" t="inlineStr">
         <is>
           <t>On-screen text</t>
         </is>
       </c>
-      <c r="B42" s="9" t="inlineStr">
-        <is>
-          <t>"i almost deleted the whole thing"  —  lower-centre</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="26" customHeight="1">
-      <c r="A43" s="20" t="inlineStr">
-        <is>
-          <t>Transition out</t>
-        </is>
-      </c>
-      <c r="B43" s="9" t="inlineStr">
-        <is>
-          <t>slow cut (breath)</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="22" customHeight="1">
-      <c r="A44" s="19" t="inlineStr">
-        <is>
-          <t>SHOT 9  ·  TURN  ·  2s  ·  SCREEN REC</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="26" customHeight="1">
-      <c r="A45" s="21" t="inlineStr">
+      <c r="B49" s="9" t="inlineStr">
+        <is>
+          <t>"i almost gave up on it"  —  lower</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="24" customHeight="1">
+      <c r="A50" s="20" t="inlineStr">
+        <is>
+          <t>Cut out</t>
+        </is>
+      </c>
+      <c r="B50" s="9" t="inlineStr">
+        <is>
+          <t>slow cut</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="19" t="inlineStr">
+        <is>
+          <t>SHOT 9  ·  TURN  ·  2s  ·  SCREEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="24" customHeight="1">
+      <c r="A53" s="21" t="inlineStr">
         <is>
           <t>Capture</t>
         </is>
       </c>
-      <c r="B45" s="13" t="inlineStr">
-        <is>
-          <t>Build SUCCEEDED</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="44" customHeight="1">
-      <c r="A46" s="21" t="inlineStr">
+      <c r="B53" s="13" t="inlineStr">
+        <is>
+          <t>Screen insert — build SUCCEEDED</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="44" customHeight="1">
+      <c r="A54" s="21" t="inlineStr">
         <is>
           <t>Do this</t>
         </is>
       </c>
-      <c r="B46" s="13" t="inlineStr">
-        <is>
-          <t>The moment it works — 'Build finished', a green check, or your QR code / install link appearing. This is the exhale.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="26" customHeight="1">
-      <c r="A47" s="21" t="inlineStr">
+      <c r="B54" s="13" t="inlineStr">
+        <is>
+          <t>'Build finished', a green check, or your QR / install link appearing. The exhale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="24" customHeight="1">
+      <c r="A55" s="21" t="inlineStr">
         <is>
           <t>On-screen text</t>
         </is>
       </c>
-      <c r="B47" s="13" t="inlineStr">
+      <c r="B55" s="13" t="inlineStr">
         <is>
           <t>"then — it built."  —  centre</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="26" customHeight="1">
-      <c r="A48" s="21" t="inlineStr">
-        <is>
-          <t>Transition out</t>
-        </is>
-      </c>
-      <c r="B48" s="13" t="inlineStr">
-        <is>
-          <t>cut on the beat</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="22" customHeight="1">
-      <c r="A49" s="19" t="inlineStr">
-        <is>
-          <t>SHOT 10  ·  TURN  ·  2s  ·  SCREEN REC / PHONE</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="26" customHeight="1">
-      <c r="A50" s="21" t="inlineStr">
+    <row r="56" ht="24" customHeight="1">
+      <c r="A56" s="21" t="inlineStr">
+        <is>
+          <t>Cut out</t>
+        </is>
+      </c>
+      <c r="B56" s="13" t="inlineStr">
+        <is>
+          <t>cut on beat</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="22" customHeight="1">
+      <c r="A58" s="19" t="inlineStr">
+        <is>
+          <t>SHOT 10  ·  TURN  ·  2s  ·  CAMERA  ·  MARK E</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="24" customHeight="1">
+      <c r="A59" s="21" t="inlineStr">
         <is>
           <t>Capture</t>
         </is>
       </c>
-      <c r="B50" s="13" t="inlineStr">
-        <is>
-          <t>Install on a real phone</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="44" customHeight="1">
-      <c r="A51" s="21" t="inlineStr">
+      <c r="B59" s="13" t="inlineStr">
+        <is>
+          <t>You + your phone — it installs</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="44" customHeight="1">
+      <c r="A60" s="21" t="inlineStr">
         <is>
           <t>Do this</t>
         </is>
       </c>
-      <c r="B51" s="13" t="inlineStr">
-        <is>
-          <t>Screen-record your phone: the APK installing, or the Memory Lane icon appearing on the home screen. Proof it's a real, shippable thing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="26" customHeight="1">
-      <c r="A52" s="21" t="inlineStr">
+      <c r="B60" s="13" t="inlineStr">
+        <is>
+          <t>You pick up your real phone; the APK installs / the app icon lands on the home screen. A small, genuine reaction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="24" customHeight="1">
+      <c r="A61" s="21" t="inlineStr">
         <is>
           <t>On-screen text</t>
         </is>
       </c>
-      <c r="B52" s="13" t="inlineStr">
-        <is>
-          <t>"it installed on a real phone"  —  top-centre</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="26" customHeight="1">
-      <c r="A53" s="21" t="inlineStr">
-        <is>
-          <t>Transition out</t>
-        </is>
-      </c>
-      <c r="B53" s="13" t="inlineStr">
+      <c r="B61" s="13" t="inlineStr">
+        <is>
+          <t>"it installed on a real phone"  —  top</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="24" customHeight="1">
+      <c r="A62" s="21" t="inlineStr">
+        <is>
+          <t>Cut out</t>
+        </is>
+      </c>
+      <c r="B62" s="13" t="inlineStr">
         <is>
           <t>hard cut</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="22" customHeight="1">
-      <c r="A54" s="19" t="inlineStr">
-        <is>
-          <t>SHOT 11  ·  GIFT  ·  4s  ·  SCREEN REC</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="26" customHeight="1">
-      <c r="A55" s="22" t="inlineStr">
+    <row r="64" ht="22" customHeight="1">
+      <c r="A64" s="19" t="inlineStr">
+        <is>
+          <t>SHOT 11  ·  GIFT  ·  4s  ·  SCREEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="24" customHeight="1">
+      <c r="A65" s="22" t="inlineStr">
         <is>
           <t>Capture</t>
         </is>
       </c>
-      <c r="B55" s="16" t="inlineStr">
-        <is>
-          <t>The app works — fill an orb</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="44" customHeight="1">
-      <c r="A56" s="22" t="inlineStr">
+      <c r="B65" s="16" t="inlineStr">
+        <is>
+          <t>Screen insert — the app WORKS</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="44" customHeight="1">
+      <c r="A66" s="22" t="inlineStr">
         <is>
           <t>Do this</t>
         </is>
       </c>
-      <c r="B56" s="16" t="inlineStr">
-        <is>
-          <t>Open Memory Lane, hold to fill an emotion, watch the orb BLEND live, let the sphere settle. The longest, calmest shot. Let it breathe.</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="26" customHeight="1">
-      <c r="A57" s="22" t="inlineStr">
+      <c r="B66" s="16" t="inlineStr">
+        <is>
+          <t>Screen-record the app: hold to fill an emotion, the orb blends live, the sphere settles. The payoff. Longest, calmest shot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="24" customHeight="1">
+      <c r="A67" s="22" t="inlineStr">
         <is>
           <t>On-screen text</t>
         </is>
       </c>
-      <c r="B57" s="16" t="inlineStr">
-        <is>
-          <t>"and it actually works"  —  top-centre</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="26" customHeight="1">
-      <c r="A58" s="22" t="inlineStr">
-        <is>
-          <t>Transition out</t>
-        </is>
-      </c>
-      <c r="B58" s="16" t="inlineStr">
+      <c r="B67" s="16" t="inlineStr">
+        <is>
+          <t>"and it actually works"  —  top</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="24" customHeight="1">
+      <c r="A68" s="22" t="inlineStr">
+        <is>
+          <t>Cut out</t>
+        </is>
+      </c>
+      <c r="B68" s="16" t="inlineStr">
         <is>
           <t>slow</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="22" customHeight="1">
-      <c r="A59" s="19" t="inlineStr">
-        <is>
-          <t>SHOT 12  ·  GIFT  ·  3s  ·  DESIGNED CARD</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="26" customHeight="1">
-      <c r="A60" s="22" t="inlineStr">
+    <row r="70" ht="22" customHeight="1">
+      <c r="A70" s="19" t="inlineStr">
+        <is>
+          <t>SHOT 12  ·  GIFT  ·  3s  ·  CAMERA  ·  MARK E</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="24" customHeight="1">
+      <c r="A71" s="22" t="inlineStr">
         <is>
           <t>Capture</t>
         </is>
       </c>
-      <c r="B60" s="16" t="inlineStr">
-        <is>
-          <t>Your handle + link over an orb</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="44" customHeight="1">
-      <c r="A61" s="22" t="inlineStr">
+      <c r="B71" s="16" t="inlineStr">
+        <is>
+          <t>You + phone, looking at it — the end</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="44" customHeight="1">
+      <c r="A72" s="22" t="inlineStr">
         <is>
           <t>Do this</t>
         </is>
       </c>
-      <c r="B61" s="16" t="inlineStr">
-        <is>
-          <t>End card: your @handle and sl1nk.com/zd015vh over a soft orb (reuse a Memory Lane frame). Hold to the end of the track.</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="26" customHeight="1">
-      <c r="A62" s="22" t="inlineStr">
+      <c r="B72" s="16" t="inlineStr">
+        <is>
+          <t>You looking down at the phone, a small real smile / relief. End card overlay: your @handle + sl1nk.com/zd015vh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="24" customHeight="1">
+      <c r="A73" s="22" t="inlineStr">
         <is>
           <t>On-screen text</t>
         </is>
       </c>
-      <c r="B62" s="16" t="inlineStr">
+      <c r="B73" s="16" t="inlineStr">
         <is>
           <t>"i built this. it's live 👇"  —  centre</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="26" customHeight="1">
-      <c r="A63" s="22" t="inlineStr">
-        <is>
-          <t>Transition out</t>
-        </is>
-      </c>
-      <c r="B63" s="16" t="inlineStr">
+    <row r="74" ht="24" customHeight="1">
+      <c r="A74" s="22" t="inlineStr">
+        <is>
+          <t>Cut out</t>
+        </is>
+      </c>
+      <c r="B74" s="16" t="inlineStr">
         <is>
           <t>hold to end</t>
         </is>
@@ -2468,16 +2800,16 @@
   </sheetData>
   <mergeCells count="12">
     <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A54:B54"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="A59:B59"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A49:B49"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A52:B52"/>
+    <mergeCell ref="A64:B64"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="A70:B70"/>
+    <mergeCell ref="A58:B58"/>
+    <mergeCell ref="A22:B22"/>
     <mergeCell ref="A34:B34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2485,6 +2817,223 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Camera Setups — the 5 tripod marks</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Set these on the tripod as you go. Lighting/outfit/body-language are on 'The Desk Shot' sheet and apply to ALL camera shots.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Mark</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Angle</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Height / distance</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Shots</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>What's in frame</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Wide, BEHIND your chair, slightly to one side</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Head height ~1.4m, 1.5-2m back</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>1, 8</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>You + the desk + the laptop glowing. The 'alone at night' establisher and the desk low-point.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Over-your-shoulder</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Just above your shoulder, ~0.6m behind</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Your hands on the keys AND the code on screen, together. Tilt slightly off-square to the screen to avoid banding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="44" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Front-ish, to one side — your face</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Eye height, ~0.8-1m</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Your face, side-lit by the screen. Watching, focused, tense. Screen out of focus behind.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="44" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Mid, side-on (profile-ish)</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Chest height, ~1.5m</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Your upper body so a lean-back / hand-drag reads. Room for the movement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="44" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Close on your hands + phone</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Eye height, ~0.6m, angled down at your hands</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>10, 12</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Your phone and your face/hands. The install, then the small smile at the end.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>THE RULE</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="44" customHeight="1">
+      <c r="A12" s="30" t="inlineStr">
+        <is>
+          <t>Camera-forward, but 3 shots MUST stay screen recordings — they're the proof and the payoff: shot 5 (the red error), shot 9 (it built), shot 11 (the orb actually blending). Everything else is you, on the tripod. A face on screen is what makes it a reel and not a screen-share.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="14"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="A12:E14"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2819,7 +3368,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3301,7 +3850,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3805,7 +4354,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4035,7 +4584,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4251,258 +4800,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Take Tracker — tick as you shoot</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Fill the yellow cells. Aim for a keeper on every shot before you start editing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Shot</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>What</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Take 1</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Take 2</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Take 3</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>Keeper?</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>Open an empty file / blank VS Code project</t>
-        </is>
-      </c>
-      <c r="C5" s="28" t="inlineStr"/>
-      <c r="D5" s="28" t="inlineStr"/>
-      <c r="E5" s="28" t="inlineStr"/>
-      <c r="F5" s="28" t="inlineStr"/>
-      <c r="G5" s="29" t="inlineStr"/>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="27" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>Your real code — scroll blend.ts / Orb.tsx</t>
-        </is>
-      </c>
-      <c r="C6" s="28" t="inlineStr"/>
-      <c r="D6" s="28" t="inlineStr"/>
-      <c r="E6" s="28" t="inlineStr"/>
-      <c r="F6" s="28" t="inlineStr"/>
-      <c r="G6" s="29" t="inlineStr"/>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="27" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>PowerShell — run the build command</t>
-        </is>
-      </c>
-      <c r="C7" s="28" t="inlineStr"/>
-      <c r="D7" s="28" t="inlineStr"/>
-      <c r="E7" s="28" t="inlineStr"/>
-      <c r="F7" s="28" t="inlineStr"/>
-      <c r="G7" s="29" t="inlineStr"/>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="27" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>EAS build logs streaming</t>
-        </is>
-      </c>
-      <c r="C8" s="28" t="inlineStr"/>
-      <c r="D8" s="28" t="inlineStr"/>
-      <c r="E8" s="28" t="inlineStr"/>
-      <c r="F8" s="28" t="inlineStr"/>
-      <c r="G8" s="29" t="inlineStr"/>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="27" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>The RED — a real / representative failure</t>
-        </is>
-      </c>
-      <c r="C9" s="28" t="inlineStr"/>
-      <c r="D9" s="28" t="inlineStr"/>
-      <c r="E9" s="28" t="inlineStr"/>
-      <c r="F9" s="28" t="inlineStr"/>
-      <c r="G9" s="29" t="inlineStr"/>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="27" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>A second, different error</t>
-        </is>
-      </c>
-      <c r="C10" s="28" t="inlineStr"/>
-      <c r="D10" s="28" t="inlineStr"/>
-      <c r="E10" s="28" t="inlineStr"/>
-      <c r="F10" s="28" t="inlineStr"/>
-      <c r="G10" s="29" t="inlineStr"/>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="27" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>git log — real late-night timestamps</t>
-        </is>
-      </c>
-      <c r="C11" s="28" t="inlineStr"/>
-      <c r="D11" s="28" t="inlineStr"/>
-      <c r="E11" s="28" t="inlineStr"/>
-      <c r="F11" s="28" t="inlineStr"/>
-      <c r="G11" s="29" t="inlineStr"/>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="27" t="n">
-        <v>8</v>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>YOU at the desk — the one human shot</t>
-        </is>
-      </c>
-      <c r="C12" s="28" t="inlineStr"/>
-      <c r="D12" s="28" t="inlineStr"/>
-      <c r="E12" s="28" t="inlineStr"/>
-      <c r="F12" s="28" t="inlineStr"/>
-      <c r="G12" s="29" t="inlineStr"/>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="27" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>Build SUCCEEDED</t>
-        </is>
-      </c>
-      <c r="C13" s="28" t="inlineStr"/>
-      <c r="D13" s="28" t="inlineStr"/>
-      <c r="E13" s="28" t="inlineStr"/>
-      <c r="F13" s="28" t="inlineStr"/>
-      <c r="G13" s="29" t="inlineStr"/>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="27" t="n">
-        <v>10</v>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>Install on a real phone</t>
-        </is>
-      </c>
-      <c r="C14" s="28" t="inlineStr"/>
-      <c r="D14" s="28" t="inlineStr"/>
-      <c r="E14" s="28" t="inlineStr"/>
-      <c r="F14" s="28" t="inlineStr"/>
-      <c r="G14" s="29" t="inlineStr"/>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="27" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>The app works — fill an orb</t>
-        </is>
-      </c>
-      <c r="C15" s="28" t="inlineStr"/>
-      <c r="D15" s="28" t="inlineStr"/>
-      <c r="E15" s="28" t="inlineStr"/>
-      <c r="F15" s="28" t="inlineStr"/>
-      <c r="G15" s="29" t="inlineStr"/>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="27" t="n">
-        <v>12</v>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>Your handle + link over an orb</t>
-        </is>
-      </c>
-      <c r="C16" s="28" t="inlineStr"/>
-      <c r="D16" s="28" t="inlineStr"/>
-      <c r="E16" s="28" t="inlineStr"/>
-      <c r="F16" s="28" t="inlineStr"/>
-      <c r="G16" s="29" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Direct every camera shot to desk-shot depth
Folds the camera guidance into one Camera Direction sheet: shared constants
(dark room, laptop-only light, dark outfit, focus lock) stated once, then a
full directed block per camera shot — frame and tripod mark, the action and
body language, the expression, and a watch-out. Notes the deliberate arc:
neutral at the start, the low point at shot 8, and the reel's only smile
saved for the final shot.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JLTsBRbD5LTCiR7DCK43kP
</commit_message>
<xml_diff>
--- a/memory-lane-reel.xlsx
+++ b/memory-lane-reel.xlsx
@@ -10,14 +10,13 @@
     <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Shot List" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Shot-by-Shot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Camera Setups" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Camera Direction" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Capture Guide" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="The Desk Shot" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Text &amp; Timing" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Edit Steps" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Music" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Take Tracker" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Post &amp; Caption" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Text &amp; Timing" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Edit Steps" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Music" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Take Tracker" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Post &amp; Caption" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -200,7 +199,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -293,6 +292,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -843,12 +851,12 @@
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>The Desk Shot</t>
+          <t>Camera Direction</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Full setup for the one human shot (shot 8): framing, lighting, what to do.</t>
+          <t>Every camera shot in full: constants (light, outfit, room) + a directed block per shot.</t>
         </is>
       </c>
     </row>
@@ -922,260 +930,6 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Take Tracker — tick as you shoot</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Fill the yellow cells. Aim for a keeper on every shot before you start editing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Shot</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>What</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Take 1</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Take 2</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Take 3</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>Keeper?</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>Open an empty file / blank VS Code project</t>
-        </is>
-      </c>
-      <c r="C5" s="28" t="inlineStr"/>
-      <c r="D5" s="28" t="inlineStr"/>
-      <c r="E5" s="28" t="inlineStr"/>
-      <c r="F5" s="28" t="inlineStr"/>
-      <c r="G5" s="29" t="inlineStr"/>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="27" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>Your real code — scroll blend.ts / Orb.tsx</t>
-        </is>
-      </c>
-      <c r="C6" s="28" t="inlineStr"/>
-      <c r="D6" s="28" t="inlineStr"/>
-      <c r="E6" s="28" t="inlineStr"/>
-      <c r="F6" s="28" t="inlineStr"/>
-      <c r="G6" s="29" t="inlineStr"/>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="27" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>PowerShell — run the build command</t>
-        </is>
-      </c>
-      <c r="C7" s="28" t="inlineStr"/>
-      <c r="D7" s="28" t="inlineStr"/>
-      <c r="E7" s="28" t="inlineStr"/>
-      <c r="F7" s="28" t="inlineStr"/>
-      <c r="G7" s="29" t="inlineStr"/>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="27" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>EAS build logs streaming</t>
-        </is>
-      </c>
-      <c r="C8" s="28" t="inlineStr"/>
-      <c r="D8" s="28" t="inlineStr"/>
-      <c r="E8" s="28" t="inlineStr"/>
-      <c r="F8" s="28" t="inlineStr"/>
-      <c r="G8" s="29" t="inlineStr"/>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="27" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>The RED — a real / representative failure</t>
-        </is>
-      </c>
-      <c r="C9" s="28" t="inlineStr"/>
-      <c r="D9" s="28" t="inlineStr"/>
-      <c r="E9" s="28" t="inlineStr"/>
-      <c r="F9" s="28" t="inlineStr"/>
-      <c r="G9" s="29" t="inlineStr"/>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="27" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>A second, different error</t>
-        </is>
-      </c>
-      <c r="C10" s="28" t="inlineStr"/>
-      <c r="D10" s="28" t="inlineStr"/>
-      <c r="E10" s="28" t="inlineStr"/>
-      <c r="F10" s="28" t="inlineStr"/>
-      <c r="G10" s="29" t="inlineStr"/>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="27" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>git log — real late-night timestamps</t>
-        </is>
-      </c>
-      <c r="C11" s="28" t="inlineStr"/>
-      <c r="D11" s="28" t="inlineStr"/>
-      <c r="E11" s="28" t="inlineStr"/>
-      <c r="F11" s="28" t="inlineStr"/>
-      <c r="G11" s="29" t="inlineStr"/>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="27" t="n">
-        <v>8</v>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>YOU at the desk — the one human shot</t>
-        </is>
-      </c>
-      <c r="C12" s="28" t="inlineStr"/>
-      <c r="D12" s="28" t="inlineStr"/>
-      <c r="E12" s="28" t="inlineStr"/>
-      <c r="F12" s="28" t="inlineStr"/>
-      <c r="G12" s="29" t="inlineStr"/>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="27" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>Build SUCCEEDED</t>
-        </is>
-      </c>
-      <c r="C13" s="28" t="inlineStr"/>
-      <c r="D13" s="28" t="inlineStr"/>
-      <c r="E13" s="28" t="inlineStr"/>
-      <c r="F13" s="28" t="inlineStr"/>
-      <c r="G13" s="29" t="inlineStr"/>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="27" t="n">
-        <v>10</v>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>Install on a real phone</t>
-        </is>
-      </c>
-      <c r="C14" s="28" t="inlineStr"/>
-      <c r="D14" s="28" t="inlineStr"/>
-      <c r="E14" s="28" t="inlineStr"/>
-      <c r="F14" s="28" t="inlineStr"/>
-      <c r="G14" s="29" t="inlineStr"/>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="27" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>The app works — fill an orb</t>
-        </is>
-      </c>
-      <c r="C15" s="28" t="inlineStr"/>
-      <c r="D15" s="28" t="inlineStr"/>
-      <c r="E15" s="28" t="inlineStr"/>
-      <c r="F15" s="28" t="inlineStr"/>
-      <c r="G15" s="29" t="inlineStr"/>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="27" t="n">
-        <v>12</v>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>Your handle + link over an orb</t>
-        </is>
-      </c>
-      <c r="C16" s="28" t="inlineStr"/>
-      <c r="D16" s="28" t="inlineStr"/>
-      <c r="E16" s="28" t="inlineStr"/>
-      <c r="F16" s="28" t="inlineStr"/>
-      <c r="G16" s="29" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2822,212 +2576,501 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:B52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="92" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Camera Setups — the 5 tripod marks</t>
+          <t>Camera Direction — every tripod shot, in full</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Set these on the tripod as you go. Lighting/outfit/body-language are on 'The Desk Shot' sheet and apply to ALL camera shots.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Mark</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Angle</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Height / distance</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Shots</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>What's in frame</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="44" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>Wide, BEHIND your chair, slightly to one side</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>Head height ~1.4m, 1.5-2m back</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>1, 8</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>You + the desk + the laptop glowing. The 'alone at night' establisher and the desk low-point.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="44" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>Over-your-shoulder</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>Just above your shoulder, ~0.6m behind</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>Your hands on the keys AND the code on screen, together. Tilt slightly off-square to the screen to avoid banding.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="44" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Front-ish, to one side — your face</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>Eye height, ~0.8-1m</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>Your face, side-lit by the screen. Watching, focused, tense. Screen out of focus behind.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="44" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Mid, side-on (profile-ish)</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>Chest height, ~1.5m</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>Your upper body so a lean-back / hand-drag reads. Room for the movement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="44" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Close on your hands + phone</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>Eye height, ~0.6m, angled down at your hands</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>10, 12</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>Your phone and your face/hands. The install, then the small smile at the end.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>THE RULE</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="44" customHeight="1">
-      <c r="A12" s="30" t="inlineStr">
-        <is>
-          <t>Camera-forward, but 3 shots MUST stay screen recordings — they're the proof and the payoff: shot 5 (the red error), shot 9 (it built), shot 11 (the orb actually blending). Everything else is you, on the tripod. A face on screen is what makes it a reel and not a screen-share.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13"/>
-    <row r="14"/>
+          <t>7 camera shots. The constants below are the same for all of them; each shot's own block covers frame, action and expression.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>CONSTANTS — true for every camera shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="35" t="inlineStr">
+        <is>
+          <t>Room</t>
+        </is>
+      </c>
+      <c r="B5" s="32" t="inlineStr">
+        <is>
+          <t>Fully dark. Curtains closed. No overhead, no lamp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="35" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="B6" s="32" t="inlineStr">
+        <is>
+          <t>ONLY the laptop screen on you. Put a bright/white screen up (light-theme editor, the logs) so it actually lights your face — a dark terminal won't. Brightness maxed, auto-brightness OFF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="35" t="inlineStr">
+        <is>
+          <t>Outfit</t>
+        </is>
+      </c>
+      <c r="B7" s="32" t="inlineStr">
+        <is>
+          <t>Same in every shot (it's one continuous night). Plain dark hoodie or tee — charcoal/black/grey. No white, no logos, no bright colours. Hoodie is ideal. Messy hair is a plus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="35" t="inlineStr">
+        <is>
+          <t>Phone / orientation</t>
+        </is>
+      </c>
+      <c r="B8" s="32" t="inlineStr">
+        <is>
+          <t>Vertical 9:16. Check the mount grips portrait. Lock focus + exposure on your face (tap-and-hold) so it doesn't hunt in the dark.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="40" customHeight="1">
+      <c r="A9" s="35" t="inlineStr">
+        <is>
+          <t>Do Not Disturb</t>
+        </is>
+      </c>
+      <c r="B9" s="32" t="inlineStr">
+        <is>
+          <t>On. No notification lights on the laptop either.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="40" customHeight="1">
+      <c r="A10" s="35" t="inlineStr">
+        <is>
+          <t>Takes</t>
+        </is>
+      </c>
+      <c r="B10" s="32" t="inlineStr">
+        <is>
+          <t>3 of each. Keep the most natural, least 'acted' one. Under-doing it always wins.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>SHOT 1 · MARK A · "3 days ago this was nothing"</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="A13" s="36" t="inlineStr">
+        <is>
+          <t>Frame &amp; tripod</t>
+        </is>
+      </c>
+      <c r="B13" s="37" t="inlineStr">
+        <is>
+          <t>Tripod WIDE, behind your chair and slightly to one side. Head height ~1.4m, 1.5-2m back. You, the desk, the laptop glowing. Top third dark for text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="42" customHeight="1">
+      <c r="A14" s="36" t="inlineStr">
+        <is>
+          <t>Do this</t>
+        </is>
+      </c>
+      <c r="B14" s="37" t="inlineStr">
+        <is>
+          <t>Start with the chair empty or you just arriving. Sit down, pull in, hands to the keyboard, settle. Calm, a beginning. Then hold 2s.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="42" customHeight="1">
+      <c r="A15" s="36" t="inlineStr">
+        <is>
+          <t>Expression</t>
+        </is>
+      </c>
+      <c r="B15" s="37" t="inlineStr">
+        <is>
+          <t>Neutral, a little hopeful. Not tired yet — this is BEFORE it all goes wrong. Save the exhaustion for later shots.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="42" customHeight="1">
+      <c r="A16" s="36" t="inlineStr">
+        <is>
+          <t>Watch out</t>
+        </is>
+      </c>
+      <c r="B16" s="37" t="inlineStr">
+        <is>
+          <t>This is your establisher — it has to read as 'one person, alone, at night, starting.' Don't rush the sit-down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>SHOT 2 · MARK B · "so i started building"</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="42" customHeight="1">
+      <c r="A19" s="36" t="inlineStr">
+        <is>
+          <t>Frame &amp; tripod</t>
+        </is>
+      </c>
+      <c r="B19" s="37" t="inlineStr">
+        <is>
+          <t>OVER YOUR SHOULDER — tripod just above/behind your shoulder, ~0.6m back, angled down. Both your hands on the keys AND the code on the screen in frame.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="42" customHeight="1">
+      <c r="A20" s="36" t="inlineStr">
+        <is>
+          <t>Do this</t>
+        </is>
+      </c>
+      <c r="B20" s="37" t="inlineStr">
+        <is>
+          <t>Actually type. Real code, real movement — a few lines, backspace, keep going. Let it look like work, not a pose.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="42" customHeight="1">
+      <c r="A21" s="36" t="inlineStr">
+        <is>
+          <t>Expression</t>
+        </is>
+      </c>
+      <c r="B21" s="37" t="inlineStr">
+        <is>
+          <t>Focused, head down. Face mostly not visible — this shot is hands + screen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="42" customHeight="1">
+      <c r="A22" s="36" t="inlineStr">
+        <is>
+          <t>Watch out</t>
+        </is>
+      </c>
+      <c r="B22" s="37" t="inlineStr">
+        <is>
+          <t>Angle slightly OFF-square to the screen so it doesn't band (those rolling dark lines). Keep the screen readable-ish but it doesn't have to be legible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>SHOT 4 · MARK C · "or so i thought"</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="42" customHeight="1">
+      <c r="A25" s="36" t="inlineStr">
+        <is>
+          <t>Frame &amp; tripod</t>
+        </is>
+      </c>
+      <c r="B25" s="37" t="inlineStr">
+        <is>
+          <t>Front-ish, to one side, on your FACE. Eye height, ~0.8-1m away. Your face side-lit by the screen; the screen soft/out of focus behind.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="42" customHeight="1">
+      <c r="A26" s="36" t="inlineStr">
+        <is>
+          <t>Do this</t>
+        </is>
+      </c>
+      <c r="B26" s="37" t="inlineStr">
+        <is>
+          <t>Watch the screen. You're waiting on the build. Small: eyes tracking, maybe lean in slightly, a slow blink. Barely anything.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="42" customHeight="1">
+      <c r="A27" s="36" t="inlineStr">
+        <is>
+          <t>Expression</t>
+        </is>
+      </c>
+      <c r="B27" s="37" t="inlineStr">
+        <is>
+          <t>Focused, a flicker of tension starting. The calm right before it breaks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="42" customHeight="1">
+      <c r="A28" s="36" t="inlineStr">
+        <is>
+          <t>Watch out</t>
+        </is>
+      </c>
+      <c r="B28" s="37" t="inlineStr">
+        <is>
+          <t>This is the setup for the error — keep it quiet so shot 5's red hits harder. Don't emote yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="19" t="inlineStr">
+        <is>
+          <t>SHOT 6 · MARK D · "and again."</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="42" customHeight="1">
+      <c r="A31" s="36" t="inlineStr">
+        <is>
+          <t>Frame &amp; tripod</t>
+        </is>
+      </c>
+      <c r="B31" s="37" t="inlineStr">
+        <is>
+          <t>Mid, side-on (profile-ish). Chest height, ~1.5m. Enough of your upper body that a lean-back and a hand movement read clearly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="42" customHeight="1">
+      <c r="A32" s="36" t="inlineStr">
+        <is>
+          <t>Do this</t>
+        </is>
+      </c>
+      <c r="B32" s="37" t="inlineStr">
+        <is>
+          <t>React to the error: lean back, drag one hand slowly down your face, OR both hands up to your head. ONE real, heavy movement. Then still.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="42" customHeight="1">
+      <c r="A33" s="36" t="inlineStr">
+        <is>
+          <t>Expression</t>
+        </is>
+      </c>
+      <c r="B33" s="37" t="inlineStr">
+        <is>
+          <t>Frustrated, deflating. Quiet defeat, not a tantrum. A sigh you can almost hear.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="42" customHeight="1">
+      <c r="A34" s="36" t="inlineStr">
+        <is>
+          <t>Watch out</t>
+        </is>
+      </c>
+      <c r="B34" s="37" t="inlineStr">
+        <is>
+          <t>One movement, slow. Two or three fidgety gestures kill it. Big acting reads fake — let the slump do the talking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="19" t="inlineStr">
+        <is>
+          <t>SHOT 8 · MARK A · "i almost gave up on it"  (the low point)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="42" customHeight="1">
+      <c r="A37" s="36" t="inlineStr">
+        <is>
+          <t>Frame &amp; tripod</t>
+        </is>
+      </c>
+      <c r="B37" s="37" t="inlineStr">
+        <is>
+          <t>Back to the WIDE behind mark (same as shot 1, so it echoes). You slumped low in the chair, the dark around you.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="42" customHeight="1">
+      <c r="A38" s="36" t="inlineStr">
+        <is>
+          <t>Do this</t>
+        </is>
+      </c>
+      <c r="B38" s="37" t="inlineStr">
+        <is>
+          <t>Do almost nothing. Slumped, head in one hand (palm on forehead / through your hair), completely still. One slow breath, maybe eyes closed for a beat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="42" customHeight="1">
+      <c r="A39" s="36" t="inlineStr">
+        <is>
+          <t>Expression</t>
+        </is>
+      </c>
+      <c r="B39" s="37" t="inlineStr">
+        <is>
+          <t>Exhausted, defeated. The emotional bottom of the whole reel. Stillness = tired; movement = acting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="42" customHeight="1">
+      <c r="A40" s="36" t="inlineStr">
+        <is>
+          <t>Watch out</t>
+        </is>
+      </c>
+      <c r="B40" s="37" t="inlineStr">
+        <is>
+          <t>Hold it a beat LONGER than feels comfortable. This is the one shot people feel. Echoing shot 1's frame (same mark) makes the fall land.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="19" t="inlineStr">
+        <is>
+          <t>SHOT 10 · MARK E · "it installed on a real phone"</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="42" customHeight="1">
+      <c r="A43" s="36" t="inlineStr">
+        <is>
+          <t>Frame &amp; tripod</t>
+        </is>
+      </c>
+      <c r="B43" s="37" t="inlineStr">
+        <is>
+          <t>Close on your HANDS + phone. Eye height, ~0.6m, angled down at your hands. Your phone clearly in frame; a bit of your face optional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="42" customHeight="1">
+      <c r="A44" s="36" t="inlineStr">
+        <is>
+          <t>Do this</t>
+        </is>
+      </c>
+      <c r="B44" s="37" t="inlineStr">
+        <is>
+          <t>Pick up your real phone, tap install / watch the app icon land on the home screen, open it. A small, genuine lift — the turn is happening.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="42" customHeight="1">
+      <c r="A45" s="36" t="inlineStr">
+        <is>
+          <t>Expression</t>
+        </is>
+      </c>
+      <c r="B45" s="37" t="inlineStr">
+        <is>
+          <t>The first real relief. A quiet 'wait… it worked?' — not a big grin yet, save that for shot 12.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="42" customHeight="1">
+      <c r="A46" s="36" t="inlineStr">
+        <is>
+          <t>Watch out</t>
+        </is>
+      </c>
+      <c r="B46" s="37" t="inlineStr">
+        <is>
+          <t>Keep the phone screen clean (DND, no clutter). This is proof it's a REAL shippable thing, so let the install actually show.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="19" t="inlineStr">
+        <is>
+          <t>SHOT 12 · MARK E · "i built this. it's live 👇"  (the end)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="42" customHeight="1">
+      <c r="A49" s="36" t="inlineStr">
+        <is>
+          <t>Frame &amp; tripod</t>
+        </is>
+      </c>
+      <c r="B49" s="37" t="inlineStr">
+        <is>
+          <t>Same close on hands + phone, or tilt up slightly to catch your face. The app open on the phone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="42" customHeight="1">
+      <c r="A50" s="36" t="inlineStr">
+        <is>
+          <t>Do this</t>
+        </is>
+      </c>
+      <c r="B50" s="37" t="inlineStr">
+        <is>
+          <t>Look down at the app running, then a small, real smile. That's it. The end card overlay (your @handle + sl1nk.com/zd015vh) sits on top.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="42" customHeight="1">
+      <c r="A51" s="36" t="inlineStr">
+        <is>
+          <t>Expression</t>
+        </is>
+      </c>
+      <c r="B51" s="37" t="inlineStr">
+        <is>
+          <t>Genuine, quiet pride. Earned relief. The payoff of the whole grind — but understated. A real half-smile beats a posed grin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="42" customHeight="1">
+      <c r="A52" s="36" t="inlineStr">
+        <is>
+          <t>Watch out</t>
+        </is>
+      </c>
+      <c r="B52" s="37" t="inlineStr">
+        <is>
+          <t>This is the ONLY smile in the reel — that's what makes it land. Don't smile in the earlier shots or this one loses its weight.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="A12:E14"/>
+  <mergeCells count="8">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A48:B48"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A12:B12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3374,488 +3417,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B50"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="84" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>The Desk Shot — shot 8, fully directed</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>The one shot you film. The emotional bottom of the reel: dark, tired, still. Everything below is set before you roll.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>1 · TRIPOD PLACEMENT</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Direction</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="38" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Where</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>BEHIND your chair, slightly to one side (in the walkway, not in front of the desk). It sees your head/shoulder and the laptop glowing in front of you.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="38" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Height</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Chest-to-eye height, ~1.2–1.5m. Level with your head — NOT high looking down (that reads like a webcam).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="38" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Distance</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>1.5–2m back. A mid shot: you, the laptop glow, dark around you. Not a close-up.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="38" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Angle</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Level or a hair down. Tilt so the TOP THIRD of frame is dark — that's where the text sits.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="38" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Orientation</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>VERTICAL 9:16. Check the mount grips portrait, not just landscape.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="38" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Lock it</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>Legs locked, mount tight. Set it once, then don't touch it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>2 · LIGHTING</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Direction</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>The only light</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>Your LAPTOP SCREEN. Turn everything else off — overhead, lamp, phone torch. Full dark except the screen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="40" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>Put a bright screen up</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>Open something white/bright (a doc, the EAS logs, VS Code light theme) so the screen actually lights your face. A dark terminal won't.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="40" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>Screen brightness</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>All the way up, and turn OFF auto-brightness so it doesn't dim mid-take.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="40" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>The look you want</t>
-        </is>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>Screen glow from below/front — cold, blue-white, a little harsh. That's the '3am, still at it' look. Perfect for this shot.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="40" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>If it's too dark</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>Phone cameras get noisy in low light. If your face is barely visible, brighten the screen or move 10cm closer — don't add a lamp, it kills the mood.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="40" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Curtains</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>Closed. No street light or daylight leaking in — it has to read as night.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>3 · OUTFIT</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>Direction</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="38" customHeight="1">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>Vibe</t>
-        </is>
-      </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>'Been at this for hours.' Comfortable, lived-in, not styled. You just don't want it to look like you dressed up for a shoot.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="38" customHeight="1">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>Best pick</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>A plain dark hoodie or a plain tee — charcoal, black, deep grey. Solid colour, no big logos or bright prints.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="38" customHeight="1">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>Avoid</t>
-        </is>
-      </c>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>Pure white (glows/blows out against the dark), bright colours, busy patterns, anything that pulls the eye off your face.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="38" customHeight="1">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>Hoodie tip</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>If you own one, a hoodie is ideal here — hood down or half-up reads 'late night grind' instantly.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="38" customHeight="1">
-      <c r="A28" s="5" t="inlineStr">
-        <is>
-          <t>Detail</t>
-        </is>
-      </c>
-      <c r="B28" s="6" t="inlineStr">
-        <is>
-          <t>Slightly messy hair is a plus, not a problem. This is the tired shot — a little dishevelled sells it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>4 · BODY LANGUAGE</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>Direction</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="36" customHeight="1">
-      <c r="A32" s="5" t="inlineStr">
-        <is>
-          <t>Overall</t>
-        </is>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
-        <is>
-          <t>Defeated, not dramatic. Heavy, slow, still. The camera should feel like it caught a real low moment, not a pose.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="36" customHeight="1">
-      <c r="A33" s="5" t="inlineStr">
-        <is>
-          <t>Shoulders</t>
-        </is>
-      </c>
-      <c r="B33" s="6" t="inlineStr">
-        <is>
-          <t>Dropped and rounded forward. Let them sink — don't sit up straight.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="36" customHeight="1">
-      <c r="A34" s="5" t="inlineStr">
-        <is>
-          <t>Head</t>
-        </is>
-      </c>
-      <c r="B34" s="6" t="inlineStr">
-        <is>
-          <t>Lowered. Either resting in one hand (palm on forehead / hand through hair) or hung down looking at the desk.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="36" customHeight="1">
-      <c r="A35" s="5" t="inlineStr">
-        <is>
-          <t>Hands</t>
-        </is>
-      </c>
-      <c r="B35" s="6" t="inlineStr">
-        <is>
-          <t>One hand up at your head OR both loose on the desk. Slow. No fidgeting, no phone, no typing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="36" customHeight="1">
-      <c r="A36" s="5" t="inlineStr">
-        <is>
-          <t>Back</t>
-        </is>
-      </c>
-      <c r="B36" s="6" t="inlineStr">
-        <is>
-          <t>Slumped low in the chair, a little curled in. Small, not upright.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="36" customHeight="1">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>Stillness</t>
-        </is>
-      </c>
-      <c r="B37" s="6" t="inlineStr">
-        <is>
-          <t>This is the whole shot. Hold nearly frozen for the full take — one slow breath, maybe one small head-shake or eyes-closed. That's it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="36" customHeight="1">
-      <c r="A38" s="5" t="inlineStr">
-        <is>
-          <t>Do NOT</t>
-        </is>
-      </c>
-      <c r="B38" s="6" t="inlineStr">
-        <is>
-          <t>Look at the camera. Smile. Move fast. Perform 'tired' with big gestures. Under-act — stillness reads as exhausted; acting reads as fake.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="22" customHeight="1">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>5 · THE 8 SECONDS</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="46" customHeight="1">
-      <c r="A41" s="30" t="inlineStr">
-        <is>
-          <t>Roll, then do almost nothing. Options, pick one: (a) sit slumped, head in hand, completely still, one slow breath; (b) rub your eyes / drag a hand down your face once, then go still; (c) stare at the screen, close your eyes for a beat, small shake of the head. Any of these, done SMALL and SLOW, is the shot. Record 3 takes and keep the stillest, most honest one. On-screen text lands here: "i almost deleted the whole thing."</t>
-        </is>
-      </c>
-    </row>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44" ht="22" customHeight="1">
-      <c r="A44" s="3" t="inlineStr">
-        <is>
-          <t>BEFORE YOU ROLL — quick check</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="22" customHeight="1">
-      <c r="A45" s="32" t="inlineStr">
-        <is>
-          <t>☐  Tripod locked, vertical, top third of frame dark</t>
-        </is>
-      </c>
-      <c r="B45" s="33" t="n"/>
-    </row>
-    <row r="46" ht="22" customHeight="1">
-      <c r="A46" s="32" t="inlineStr">
-        <is>
-          <t>☐  Every light off except the laptop; bright screen up; brightness maxed, auto-brightness off</t>
-        </is>
-      </c>
-      <c r="B46" s="33" t="n"/>
-    </row>
-    <row r="47" ht="22" customHeight="1">
-      <c r="A47" s="32" t="inlineStr">
-        <is>
-          <t>☐  Curtains closed</t>
-        </is>
-      </c>
-      <c r="B47" s="33" t="n"/>
-    </row>
-    <row r="48" ht="22" customHeight="1">
-      <c r="A48" s="32" t="inlineStr">
-        <is>
-          <t>☐  Dark plain outfit on</t>
-        </is>
-      </c>
-      <c r="B48" s="33" t="n"/>
-    </row>
-    <row r="49" ht="22" customHeight="1">
-      <c r="A49" s="32" t="inlineStr">
-        <is>
-          <t>☐  Do Not Disturb on; no notification lights</t>
-        </is>
-      </c>
-      <c r="B49" s="33" t="n"/>
-    </row>
-    <row r="50" ht="22" customHeight="1">
-      <c r="A50" s="32" t="inlineStr">
-        <is>
-          <t>☐  Focus + exposure locked on your face</t>
-        </is>
-      </c>
-      <c r="B50" s="33" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="13">
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A48:B48"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="A49:B49"/>
-    <mergeCell ref="A47:B47"/>
-    <mergeCell ref="A41:B43"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A50:B50"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -4354,7 +3915,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4584,7 +4145,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4800,4 +4361,258 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Take Tracker — tick as you shoot</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Fill the yellow cells. Aim for a keeper on every shot before you start editing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Shot</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>What</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Take 1</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Take 2</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Take 3</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Keeper?</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Open an empty file / blank VS Code project</t>
+        </is>
+      </c>
+      <c r="C5" s="28" t="inlineStr"/>
+      <c r="D5" s="28" t="inlineStr"/>
+      <c r="E5" s="28" t="inlineStr"/>
+      <c r="F5" s="28" t="inlineStr"/>
+      <c r="G5" s="29" t="inlineStr"/>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Your real code — scroll blend.ts / Orb.tsx</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="inlineStr"/>
+      <c r="D6" s="28" t="inlineStr"/>
+      <c r="E6" s="28" t="inlineStr"/>
+      <c r="F6" s="28" t="inlineStr"/>
+      <c r="G6" s="29" t="inlineStr"/>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>PowerShell — run the build command</t>
+        </is>
+      </c>
+      <c r="C7" s="28" t="inlineStr"/>
+      <c r="D7" s="28" t="inlineStr"/>
+      <c r="E7" s="28" t="inlineStr"/>
+      <c r="F7" s="28" t="inlineStr"/>
+      <c r="G7" s="29" t="inlineStr"/>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="27" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>EAS build logs streaming</t>
+        </is>
+      </c>
+      <c r="C8" s="28" t="inlineStr"/>
+      <c r="D8" s="28" t="inlineStr"/>
+      <c r="E8" s="28" t="inlineStr"/>
+      <c r="F8" s="28" t="inlineStr"/>
+      <c r="G8" s="29" t="inlineStr"/>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="27" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>The RED — a real / representative failure</t>
+        </is>
+      </c>
+      <c r="C9" s="28" t="inlineStr"/>
+      <c r="D9" s="28" t="inlineStr"/>
+      <c r="E9" s="28" t="inlineStr"/>
+      <c r="F9" s="28" t="inlineStr"/>
+      <c r="G9" s="29" t="inlineStr"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="27" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>A second, different error</t>
+        </is>
+      </c>
+      <c r="C10" s="28" t="inlineStr"/>
+      <c r="D10" s="28" t="inlineStr"/>
+      <c r="E10" s="28" t="inlineStr"/>
+      <c r="F10" s="28" t="inlineStr"/>
+      <c r="G10" s="29" t="inlineStr"/>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="27" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>git log — real late-night timestamps</t>
+        </is>
+      </c>
+      <c r="C11" s="28" t="inlineStr"/>
+      <c r="D11" s="28" t="inlineStr"/>
+      <c r="E11" s="28" t="inlineStr"/>
+      <c r="F11" s="28" t="inlineStr"/>
+      <c r="G11" s="29" t="inlineStr"/>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="27" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>YOU at the desk — the one human shot</t>
+        </is>
+      </c>
+      <c r="C12" s="28" t="inlineStr"/>
+      <c r="D12" s="28" t="inlineStr"/>
+      <c r="E12" s="28" t="inlineStr"/>
+      <c r="F12" s="28" t="inlineStr"/>
+      <c r="G12" s="29" t="inlineStr"/>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="27" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Build SUCCEEDED</t>
+        </is>
+      </c>
+      <c r="C13" s="28" t="inlineStr"/>
+      <c r="D13" s="28" t="inlineStr"/>
+      <c r="E13" s="28" t="inlineStr"/>
+      <c r="F13" s="28" t="inlineStr"/>
+      <c r="G13" s="29" t="inlineStr"/>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="27" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Install on a real phone</t>
+        </is>
+      </c>
+      <c r="C14" s="28" t="inlineStr"/>
+      <c r="D14" s="28" t="inlineStr"/>
+      <c r="E14" s="28" t="inlineStr"/>
+      <c r="F14" s="28" t="inlineStr"/>
+      <c r="G14" s="29" t="inlineStr"/>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="27" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>The app works — fill an orb</t>
+        </is>
+      </c>
+      <c r="C15" s="28" t="inlineStr"/>
+      <c r="D15" s="28" t="inlineStr"/>
+      <c r="E15" s="28" t="inlineStr"/>
+      <c r="F15" s="28" t="inlineStr"/>
+      <c r="G15" s="29" t="inlineStr"/>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="27" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Your handle + link over an orb</t>
+        </is>
+      </c>
+      <c r="C16" s="28" t="inlineStr"/>
+      <c r="D16" s="28" t="inlineStr"/>
+      <c r="E16" s="28" t="inlineStr"/>
+      <c r="F16" s="28" t="inlineStr"/>
+      <c r="G16" s="29" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>